<commit_message>
Map part primary flags from SPI main alternatives
</commit_message>
<xml_diff>
--- a/docs/field-map/CoCre8_PlanningV2_Template_Field_Map.xlsx
+++ b/docs/field-map/CoCre8_PlanningV2_Template_Field_Map.xlsx
@@ -18,7 +18,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Target Fields'!$A$1:$P$153</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Template Fields'!$A$1:$H$180</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Source Evidence'!$A$1:$D$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Unknowns'!$A$1:$G$268</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Unknowns'!$A$1:$G$266</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Output Objects'!$A$1:$E$34</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'SAP Investigation Log'!$A$1:$E$10</definedName>
   </definedNames>
@@ -231,8 +231,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Unknowns" displayName="Unknowns" ref="A1:G268" headerRowCount="1">
-  <autoFilter ref="A1:G268"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Unknowns" displayName="Unknowns" ref="A1:G266" headerRowCount="1">
+  <autoFilter ref="A1:G266"/>
   <tableColumns count="7">
     <tableColumn id="1" name="Field"/>
     <tableColumn id="2" name="Object"/>
@@ -12409,7 +12409,7 @@
     <col width="23" customWidth="1" min="3" max="3"/>
     <col width="62" customWidth="1" min="4" max="4"/>
     <col width="23" customWidth="1" min="5" max="5"/>
-    <col width="51" customWidth="1" min="6" max="6"/>
+    <col width="62" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="62" customWidth="1" min="8" max="8"/>
   </cols>
@@ -13055,70 +13055,78 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="4" t="inlineStr">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>Parts</t>
         </is>
       </c>
-      <c r="B19" s="4" t="inlineStr">
+      <c r="B19" s="2" t="inlineStr">
         <is>
           <t>isPrimary</t>
         </is>
       </c>
-      <c r="C19" s="4" t="inlineStr">
+      <c r="C19" s="2" t="inlineStr">
         <is>
           <t>Boolean</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr"/>
-      <c r="E19" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F19" s="4" t="inlineStr"/>
-      <c r="G19" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H19" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+      <c r="D19" s="2" t="inlineStr"/>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>SPI_DATA.csv:Main alternative par equals material/part number</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>Populated from SPI_DATA.csv Main alternative par. Blank when SPI has no main alternative value.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="4" t="inlineStr">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>Parts</t>
         </is>
       </c>
-      <c r="B20" s="4" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>primaryPartNumber</t>
         </is>
       </c>
-      <c r="C20" s="4" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr">
         <is>
           <t>String</t>
         </is>
       </c>
-      <c r="D20" s="4" t="inlineStr"/>
-      <c r="E20" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F20" s="4" t="inlineStr"/>
-      <c r="G20" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H20" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+      <c r="D20" s="2" t="inlineStr"/>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>SPI_DATA.csv:Main alternative par</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>Populated from SPI_DATA.csv Main alternative par. Blank when SPI has no main alternative value.</t>
         </is>
       </c>
     </row>
@@ -13194,7 +13202,7 @@
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+          <t>Left blank. User indicated this field is unlikely to be available from current CoCre8 sources.</t>
         </is>
       </c>
     </row>
@@ -13232,7 +13240,7 @@
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+          <t>Left blank. User indicated this field is unlikely to be available from current CoCre8 sources.</t>
         </is>
       </c>
     </row>
@@ -13266,7 +13274,7 @@
       </c>
       <c r="H24" s="4" t="inlineStr">
         <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+          <t>Left blank. CoCre8 local reporting has only item group codes; live SAP ItemGroups/OITM needs investigation for class/type semantics.</t>
         </is>
       </c>
     </row>
@@ -13300,7 +13308,7 @@
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+          <t>Left blank. CoCre8 local reporting has only item group codes; live SAP ItemGroups/OITM needs investigation for class/type semantics.</t>
         </is>
       </c>
     </row>
@@ -13334,7 +13342,7 @@
       </c>
       <c r="H26" s="4" t="inlineStr">
         <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+          <t>Left blank. User indicated this field is unlikely to be available from current CoCre8 sources.</t>
         </is>
       </c>
     </row>
@@ -13368,7 +13376,7 @@
       </c>
       <c r="H27" s="4" t="inlineStr">
         <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+          <t>Left blank. CoCre8 local reporting has only item group codes; live SAP ItemGroups/OITM needs investigation for class/type semantics.</t>
         </is>
       </c>
     </row>
@@ -13402,7 +13410,7 @@
       </c>
       <c r="H28" s="4" t="inlineStr">
         <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+          <t>Left blank. User indicated this field is unlikely to be available from current CoCre8 sources.</t>
         </is>
       </c>
     </row>
@@ -13436,7 +13444,7 @@
       </c>
       <c r="H29" s="4" t="inlineStr">
         <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+          <t>Left blank. User indicated this field is unlikely to be available from current CoCre8 sources.</t>
         </is>
       </c>
     </row>
@@ -13470,7 +13478,7 @@
       </c>
       <c r="H30" s="4" t="inlineStr">
         <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+          <t>Left blank. User indicated this field is unlikely to be available from current CoCre8 sources.</t>
         </is>
       </c>
     </row>
@@ -13504,7 +13512,7 @@
       </c>
       <c r="H31" s="4" t="inlineStr">
         <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+          <t>Left blank. User indicated this field is unlikely to be available from current CoCre8 sources.</t>
         </is>
       </c>
     </row>
@@ -13538,7 +13546,7 @@
       </c>
       <c r="H32" s="4" t="inlineStr">
         <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+          <t>Left blank. User indicated this field is unlikely to be available from current CoCre8 sources.</t>
         </is>
       </c>
     </row>
@@ -13572,7 +13580,7 @@
       </c>
       <c r="H33" s="4" t="inlineStr">
         <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+          <t>Left blank. User indicated this field is unlikely to be available from current CoCre8 sources.</t>
         </is>
       </c>
     </row>
@@ -13610,7 +13618,7 @@
       </c>
       <c r="H34" s="4" t="inlineStr">
         <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+          <t>Left blank. User indicated this field is unlikely to be available from current CoCre8 sources.</t>
         </is>
       </c>
     </row>
@@ -13648,7 +13656,7 @@
       </c>
       <c r="H35" s="4" t="inlineStr">
         <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+          <t>Left blank. User indicated this field is unlikely to be available from current CoCre8 sources.</t>
         </is>
       </c>
     </row>
@@ -18961,7 +18969,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G268"/>
+  <dimension ref="A1:G266"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -23231,7 +23239,7 @@
     <row r="116">
       <c r="A116" s="4" t="inlineStr">
         <is>
-          <t>isPrimary</t>
+          <t>isBranchStockable</t>
         </is>
       </c>
       <c r="B116" s="4" t="inlineStr">
@@ -23251,7 +23259,7 @@
       </c>
       <c r="E116" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Parts.isPrimary?</t>
+          <t>What confirmed CoCre8/SAP source should populate Parts.isBranchStockable?</t>
         </is>
       </c>
       <c r="F116" s="4" t="inlineStr">
@@ -23261,14 +23269,14 @@
       </c>
       <c r="G116" s="4" t="inlineStr">
         <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+          <t>Left blank. User indicated this field is unlikely to be available from current CoCre8 sources.</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="4" t="inlineStr">
         <is>
-          <t>primaryPartNumber</t>
+          <t>isBootStockable</t>
         </is>
       </c>
       <c r="B117" s="4" t="inlineStr">
@@ -23288,7 +23296,7 @@
       </c>
       <c r="E117" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Parts.primaryPartNumber?</t>
+          <t>What confirmed CoCre8/SAP source should populate Parts.isBootStockable?</t>
         </is>
       </c>
       <c r="F117" s="4" t="inlineStr">
@@ -23298,14 +23306,14 @@
       </c>
       <c r="G117" s="4" t="inlineStr">
         <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+          <t>Left blank. User indicated this field is unlikely to be available from current CoCre8 sources.</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="4" t="inlineStr">
         <is>
-          <t>isBranchStockable</t>
+          <t>productClass</t>
         </is>
       </c>
       <c r="B118" s="4" t="inlineStr">
@@ -23325,7 +23333,7 @@
       </c>
       <c r="E118" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Parts.isBranchStockable?</t>
+          <t>What confirmed CoCre8/SAP source should populate Parts.productClass?</t>
         </is>
       </c>
       <c r="F118" s="4" t="inlineStr">
@@ -23335,14 +23343,14 @@
       </c>
       <c r="G118" s="4" t="inlineStr">
         <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+          <t>Left blank. CoCre8 local reporting has only item group codes; live SAP ItemGroups/OITM needs investigation for class/type semantics.</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="4" t="inlineStr">
         <is>
-          <t>isBootStockable</t>
+          <t>productType</t>
         </is>
       </c>
       <c r="B119" s="4" t="inlineStr">
@@ -23362,7 +23370,7 @@
       </c>
       <c r="E119" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Parts.isBootStockable?</t>
+          <t>What confirmed CoCre8/SAP source should populate Parts.productType?</t>
         </is>
       </c>
       <c r="F119" s="4" t="inlineStr">
@@ -23372,14 +23380,14 @@
       </c>
       <c r="G119" s="4" t="inlineStr">
         <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+          <t>Left blank. CoCre8 local reporting has only item group codes; live SAP ItemGroups/OITM needs investigation for class/type semantics.</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="4" t="inlineStr">
         <is>
-          <t>productClass</t>
+          <t>costCategory</t>
         </is>
       </c>
       <c r="B120" s="4" t="inlineStr">
@@ -23399,7 +23407,7 @@
       </c>
       <c r="E120" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Parts.productClass?</t>
+          <t>What confirmed CoCre8/SAP source should populate Parts.costCategory?</t>
         </is>
       </c>
       <c r="F120" s="4" t="inlineStr">
@@ -23409,14 +23417,14 @@
       </c>
       <c r="G120" s="4" t="inlineStr">
         <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+          <t>Left blank. User indicated this field is unlikely to be available from current CoCre8 sources.</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="4" t="inlineStr">
         <is>
-          <t>productType</t>
+          <t>partType</t>
         </is>
       </c>
       <c r="B121" s="4" t="inlineStr">
@@ -23436,7 +23444,7 @@
       </c>
       <c r="E121" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Parts.productType?</t>
+          <t>What confirmed CoCre8/SAP source should populate Parts.partType?</t>
         </is>
       </c>
       <c r="F121" s="4" t="inlineStr">
@@ -23446,14 +23454,14 @@
       </c>
       <c r="G121" s="4" t="inlineStr">
         <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+          <t>Left blank. CoCre8 local reporting has only item group codes; live SAP ItemGroups/OITM needs investigation for class/type semantics.</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="4" t="inlineStr">
         <is>
-          <t>costCategory</t>
+          <t>isKit</t>
         </is>
       </c>
       <c r="B122" s="4" t="inlineStr">
@@ -23473,7 +23481,7 @@
       </c>
       <c r="E122" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Parts.costCategory?</t>
+          <t>What confirmed CoCre8/SAP source should populate Parts.isKit?</t>
         </is>
       </c>
       <c r="F122" s="4" t="inlineStr">
@@ -23483,14 +23491,14 @@
       </c>
       <c r="G122" s="4" t="inlineStr">
         <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+          <t>Left blank. User indicated this field is unlikely to be available from current CoCre8 sources.</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="4" t="inlineStr">
         <is>
-          <t>partType</t>
+          <t>isObsolete</t>
         </is>
       </c>
       <c r="B123" s="4" t="inlineStr">
@@ -23510,7 +23518,7 @@
       </c>
       <c r="E123" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Parts.partType?</t>
+          <t>What confirmed CoCre8/SAP source should populate Parts.isObsolete?</t>
         </is>
       </c>
       <c r="F123" s="4" t="inlineStr">
@@ -23520,14 +23528,14 @@
       </c>
       <c r="G123" s="4" t="inlineStr">
         <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+          <t>Left blank. User indicated this field is unlikely to be available from current CoCre8 sources.</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="4" t="inlineStr">
         <is>
-          <t>isKit</t>
+          <t>isService</t>
         </is>
       </c>
       <c r="B124" s="4" t="inlineStr">
@@ -23547,7 +23555,7 @@
       </c>
       <c r="E124" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Parts.isKit?</t>
+          <t>What confirmed CoCre8/SAP source should populate Parts.isService?</t>
         </is>
       </c>
       <c r="F124" s="4" t="inlineStr">
@@ -23557,14 +23565,14 @@
       </c>
       <c r="G124" s="4" t="inlineStr">
         <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+          <t>Left blank. User indicated this field is unlikely to be available from current CoCre8 sources.</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="4" t="inlineStr">
         <is>
-          <t>isObsolete</t>
+          <t>isTool</t>
         </is>
       </c>
       <c r="B125" s="4" t="inlineStr">
@@ -23584,7 +23592,7 @@
       </c>
       <c r="E125" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Parts.isObsolete?</t>
+          <t>What confirmed CoCre8/SAP source should populate Parts.isTool?</t>
         </is>
       </c>
       <c r="F125" s="4" t="inlineStr">
@@ -23594,14 +23602,14 @@
       </c>
       <c r="G125" s="4" t="inlineStr">
         <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+          <t>Left blank. User indicated this field is unlikely to be available from current CoCre8 sources.</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="4" t="inlineStr">
         <is>
-          <t>isService</t>
+          <t>isExcludeFromReplenishment</t>
         </is>
       </c>
       <c r="B126" s="4" t="inlineStr">
@@ -23621,7 +23629,7 @@
       </c>
       <c r="E126" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Parts.isService?</t>
+          <t>What confirmed CoCre8/SAP source should populate Parts.isExcludeFromReplenishment?</t>
         </is>
       </c>
       <c r="F126" s="4" t="inlineStr">
@@ -23631,14 +23639,14 @@
       </c>
       <c r="G126" s="4" t="inlineStr">
         <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+          <t>Left blank. User indicated this field is unlikely to be available from current CoCre8 sources.</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="4" t="inlineStr">
         <is>
-          <t>isTool</t>
+          <t>isSmallPart</t>
         </is>
       </c>
       <c r="B127" s="4" t="inlineStr">
@@ -23658,7 +23666,7 @@
       </c>
       <c r="E127" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Parts.isTool?</t>
+          <t>What confirmed CoCre8/SAP source should populate Parts.isSmallPart?</t>
         </is>
       </c>
       <c r="F127" s="4" t="inlineStr">
@@ -23668,14 +23676,14 @@
       </c>
       <c r="G127" s="4" t="inlineStr">
         <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+          <t>Left blank. User indicated this field is unlikely to be available from current CoCre8 sources.</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="4" t="inlineStr">
         <is>
-          <t>isExcludeFromReplenishment</t>
+          <t>purchaseLeadTimeDays</t>
         </is>
       </c>
       <c r="B128" s="4" t="inlineStr">
@@ -23695,7 +23703,7 @@
       </c>
       <c r="E128" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Parts.isExcludeFromReplenishment?</t>
+          <t>What confirmed CoCre8/SAP source should populate Parts.purchaseLeadTimeDays?</t>
         </is>
       </c>
       <c r="F128" s="4" t="inlineStr">
@@ -23705,14 +23713,14 @@
       </c>
       <c r="G128" s="4" t="inlineStr">
         <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+          <t>Left blank. User indicated this field is unlikely to be available from current CoCre8 sources.</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="4" t="inlineStr">
         <is>
-          <t>isSmallPart</t>
+          <t>isCritical</t>
         </is>
       </c>
       <c r="B129" s="4" t="inlineStr">
@@ -23732,7 +23740,7 @@
       </c>
       <c r="E129" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Parts.isSmallPart?</t>
+          <t>What confirmed CoCre8/SAP source should populate Parts.isCritical?</t>
         </is>
       </c>
       <c r="F129" s="4" t="inlineStr">
@@ -23742,19 +23750,19 @@
       </c>
       <c r="G129" s="4" t="inlineStr">
         <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+          <t>Left blank. User indicated this field is unlikely to be available from current CoCre8 sources.</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="4" t="inlineStr">
         <is>
-          <t>purchaseLeadTimeDays</t>
+          <t>externalAddressId</t>
         </is>
       </c>
       <c r="B130" s="4" t="inlineStr">
         <is>
-          <t>Parts</t>
+          <t>Addresses</t>
         </is>
       </c>
       <c r="C130" s="4" t="inlineStr">
@@ -23769,7 +23777,7 @@
       </c>
       <c r="E130" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Parts.purchaseLeadTimeDays?</t>
+          <t>What confirmed CoCre8/SAP source should populate Addresses.externalAddressId?</t>
         </is>
       </c>
       <c r="F130" s="4" t="inlineStr">
@@ -23786,12 +23794,12 @@
     <row r="131">
       <c r="A131" s="4" t="inlineStr">
         <is>
-          <t>isCritical</t>
+          <t>customerExternalId</t>
         </is>
       </c>
       <c r="B131" s="4" t="inlineStr">
         <is>
-          <t>Parts</t>
+          <t>Addresses</t>
         </is>
       </c>
       <c r="C131" s="4" t="inlineStr">
@@ -23806,7 +23814,7 @@
       </c>
       <c r="E131" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Parts.isCritical?</t>
+          <t>What confirmed CoCre8/SAP source should populate Addresses.customerExternalId?</t>
         </is>
       </c>
       <c r="F131" s="4" t="inlineStr">
@@ -23823,7 +23831,7 @@
     <row r="132">
       <c r="A132" s="4" t="inlineStr">
         <is>
-          <t>externalAddressId</t>
+          <t>addressLine1</t>
         </is>
       </c>
       <c r="B132" s="4" t="inlineStr">
@@ -23843,7 +23851,7 @@
       </c>
       <c r="E132" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Addresses.externalAddressId?</t>
+          <t>What confirmed CoCre8/SAP source should populate Addresses.addressLine1?</t>
         </is>
       </c>
       <c r="F132" s="4" t="inlineStr">
@@ -23860,7 +23868,7 @@
     <row r="133">
       <c r="A133" s="4" t="inlineStr">
         <is>
-          <t>customerExternalId</t>
+          <t>addressLine2</t>
         </is>
       </c>
       <c r="B133" s="4" t="inlineStr">
@@ -23880,7 +23888,7 @@
       </c>
       <c r="E133" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Addresses.customerExternalId?</t>
+          <t>What confirmed CoCre8/SAP source should populate Addresses.addressLine2?</t>
         </is>
       </c>
       <c r="F133" s="4" t="inlineStr">
@@ -23897,7 +23905,7 @@
     <row r="134">
       <c r="A134" s="4" t="inlineStr">
         <is>
-          <t>addressLine1</t>
+          <t>addressLine3</t>
         </is>
       </c>
       <c r="B134" s="4" t="inlineStr">
@@ -23917,7 +23925,7 @@
       </c>
       <c r="E134" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Addresses.addressLine1?</t>
+          <t>What confirmed CoCre8/SAP source should populate Addresses.addressLine3?</t>
         </is>
       </c>
       <c r="F134" s="4" t="inlineStr">
@@ -23934,7 +23942,7 @@
     <row r="135">
       <c r="A135" s="4" t="inlineStr">
         <is>
-          <t>addressLine2</t>
+          <t>city</t>
         </is>
       </c>
       <c r="B135" s="4" t="inlineStr">
@@ -23954,7 +23962,7 @@
       </c>
       <c r="E135" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Addresses.addressLine2?</t>
+          <t>What confirmed CoCre8/SAP source should populate Addresses.city?</t>
         </is>
       </c>
       <c r="F135" s="4" t="inlineStr">
@@ -23971,7 +23979,7 @@
     <row r="136">
       <c r="A136" s="4" t="inlineStr">
         <is>
-          <t>addressLine3</t>
+          <t>stateProvince</t>
         </is>
       </c>
       <c r="B136" s="4" t="inlineStr">
@@ -23991,7 +23999,7 @@
       </c>
       <c r="E136" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Addresses.addressLine3?</t>
+          <t>What confirmed CoCre8/SAP source should populate Addresses.stateProvince?</t>
         </is>
       </c>
       <c r="F136" s="4" t="inlineStr">
@@ -24008,7 +24016,7 @@
     <row r="137">
       <c r="A137" s="4" t="inlineStr">
         <is>
-          <t>city</t>
+          <t>countryCode</t>
         </is>
       </c>
       <c r="B137" s="4" t="inlineStr">
@@ -24028,7 +24036,7 @@
       </c>
       <c r="E137" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Addresses.city?</t>
+          <t>What confirmed CoCre8/SAP source should populate Addresses.countryCode?</t>
         </is>
       </c>
       <c r="F137" s="4" t="inlineStr">
@@ -24045,7 +24053,7 @@
     <row r="138">
       <c r="A138" s="4" t="inlineStr">
         <is>
-          <t>stateProvince</t>
+          <t>latitude</t>
         </is>
       </c>
       <c r="B138" s="4" t="inlineStr">
@@ -24065,7 +24073,7 @@
       </c>
       <c r="E138" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Addresses.stateProvince?</t>
+          <t>What confirmed CoCre8/SAP source should populate Addresses.latitude?</t>
         </is>
       </c>
       <c r="F138" s="4" t="inlineStr">
@@ -24082,7 +24090,7 @@
     <row r="139">
       <c r="A139" s="4" t="inlineStr">
         <is>
-          <t>countryCode</t>
+          <t>longitude</t>
         </is>
       </c>
       <c r="B139" s="4" t="inlineStr">
@@ -24102,7 +24110,7 @@
       </c>
       <c r="E139" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Addresses.countryCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate Addresses.longitude?</t>
         </is>
       </c>
       <c r="F139" s="4" t="inlineStr">
@@ -24119,7 +24127,7 @@
     <row r="140">
       <c r="A140" s="4" t="inlineStr">
         <is>
-          <t>latitude</t>
+          <t>timeZone</t>
         </is>
       </c>
       <c r="B140" s="4" t="inlineStr">
@@ -24139,7 +24147,7 @@
       </c>
       <c r="E140" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Addresses.latitude?</t>
+          <t>What confirmed CoCre8/SAP source should populate Addresses.timeZone?</t>
         </is>
       </c>
       <c r="F140" s="4" t="inlineStr">
@@ -24156,7 +24164,7 @@
     <row r="141">
       <c r="A141" s="4" t="inlineStr">
         <is>
-          <t>longitude</t>
+          <t>nodeId</t>
         </is>
       </c>
       <c r="B141" s="4" t="inlineStr">
@@ -24176,7 +24184,7 @@
       </c>
       <c r="E141" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Addresses.longitude?</t>
+          <t>What confirmed CoCre8/SAP source should populate Addresses.nodeId?</t>
         </is>
       </c>
       <c r="F141" s="4" t="inlineStr">
@@ -24193,12 +24201,12 @@
     <row r="142">
       <c r="A142" s="4" t="inlineStr">
         <is>
-          <t>timeZone</t>
+          <t>addressId</t>
         </is>
       </c>
       <c r="B142" s="4" t="inlineStr">
         <is>
-          <t>Addresses</t>
+          <t>Warehouses</t>
         </is>
       </c>
       <c r="C142" s="4" t="inlineStr">
@@ -24213,7 +24221,7 @@
       </c>
       <c r="E142" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Addresses.timeZone?</t>
+          <t>What confirmed CoCre8/SAP source should populate Warehouses.addressId?</t>
         </is>
       </c>
       <c r="F142" s="4" t="inlineStr">
@@ -24235,7 +24243,7 @@
       </c>
       <c r="B143" s="4" t="inlineStr">
         <is>
-          <t>Addresses</t>
+          <t>Warehouses</t>
         </is>
       </c>
       <c r="C143" s="4" t="inlineStr">
@@ -24250,7 +24258,7 @@
       </c>
       <c r="E143" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Addresses.nodeId?</t>
+          <t>What confirmed CoCre8/SAP source should populate Warehouses.nodeId?</t>
         </is>
       </c>
       <c r="F143" s="4" t="inlineStr">
@@ -24267,7 +24275,7 @@
     <row r="144">
       <c r="A144" s="4" t="inlineStr">
         <is>
-          <t>addressId</t>
+          <t>returnWarehouseId</t>
         </is>
       </c>
       <c r="B144" s="4" t="inlineStr">
@@ -24287,7 +24295,7 @@
       </c>
       <c r="E144" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Warehouses.addressId?</t>
+          <t>What confirmed CoCre8/SAP source should populate Warehouses.returnWarehouseId?</t>
         </is>
       </c>
       <c r="F144" s="4" t="inlineStr">
@@ -24304,7 +24312,7 @@
     <row r="145">
       <c r="A145" s="4" t="inlineStr">
         <is>
-          <t>nodeId</t>
+          <t>supplyWarehouseId</t>
         </is>
       </c>
       <c r="B145" s="4" t="inlineStr">
@@ -24324,7 +24332,7 @@
       </c>
       <c r="E145" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Warehouses.nodeId?</t>
+          <t>What confirmed CoCre8/SAP source should populate Warehouses.supplyWarehouseId?</t>
         </is>
       </c>
       <c r="F145" s="4" t="inlineStr">
@@ -24341,7 +24349,7 @@
     <row r="146">
       <c r="A146" s="4" t="inlineStr">
         <is>
-          <t>returnWarehouseId</t>
+          <t>warehouseTypeId</t>
         </is>
       </c>
       <c r="B146" s="4" t="inlineStr">
@@ -24361,7 +24369,7 @@
       </c>
       <c r="E146" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Warehouses.returnWarehouseId?</t>
+          <t>What confirmed CoCre8/SAP source should populate Warehouses.warehouseTypeId?</t>
         </is>
       </c>
       <c r="F146" s="4" t="inlineStr">
@@ -24378,7 +24386,7 @@
     <row r="147">
       <c r="A147" s="4" t="inlineStr">
         <is>
-          <t>supplyWarehouseId</t>
+          <t>isRepairWarehouse</t>
         </is>
       </c>
       <c r="B147" s="4" t="inlineStr">
@@ -24398,7 +24406,7 @@
       </c>
       <c r="E147" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Warehouses.supplyWarehouseId?</t>
+          <t>What confirmed CoCre8/SAP source should populate Warehouses.isRepairWarehouse?</t>
         </is>
       </c>
       <c r="F147" s="4" t="inlineStr">
@@ -24415,7 +24423,7 @@
     <row r="148">
       <c r="A148" s="4" t="inlineStr">
         <is>
-          <t>warehouseTypeId</t>
+          <t>isReplenishable</t>
         </is>
       </c>
       <c r="B148" s="4" t="inlineStr">
@@ -24435,7 +24443,7 @@
       </c>
       <c r="E148" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Warehouses.warehouseTypeId?</t>
+          <t>What confirmed CoCre8/SAP source should populate Warehouses.isReplenishable?</t>
         </is>
       </c>
       <c r="F148" s="4" t="inlineStr">
@@ -24452,7 +24460,7 @@
     <row r="149">
       <c r="A149" s="4" t="inlineStr">
         <is>
-          <t>isRepairWarehouse</t>
+          <t>isBootStockable</t>
         </is>
       </c>
       <c r="B149" s="4" t="inlineStr">
@@ -24472,7 +24480,7 @@
       </c>
       <c r="E149" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Warehouses.isRepairWarehouse?</t>
+          <t>What confirmed CoCre8/SAP source should populate Warehouses.isBootStockable?</t>
         </is>
       </c>
       <c r="F149" s="4" t="inlineStr">
@@ -24489,7 +24497,7 @@
     <row r="150">
       <c r="A150" s="4" t="inlineStr">
         <is>
-          <t>isReplenishable</t>
+          <t>isBranchStockable</t>
         </is>
       </c>
       <c r="B150" s="4" t="inlineStr">
@@ -24509,7 +24517,7 @@
       </c>
       <c r="E150" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Warehouses.isReplenishable?</t>
+          <t>What confirmed CoCre8/SAP source should populate Warehouses.isBranchStockable?</t>
         </is>
       </c>
       <c r="F150" s="4" t="inlineStr">
@@ -24526,7 +24534,7 @@
     <row r="151">
       <c r="A151" s="4" t="inlineStr">
         <is>
-          <t>isBootStockable</t>
+          <t>isRemote</t>
         </is>
       </c>
       <c r="B151" s="4" t="inlineStr">
@@ -24546,7 +24554,7 @@
       </c>
       <c r="E151" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Warehouses.isBootStockable?</t>
+          <t>What confirmed CoCre8/SAP source should populate Warehouses.isRemote?</t>
         </is>
       </c>
       <c r="F151" s="4" t="inlineStr">
@@ -24563,7 +24571,7 @@
     <row r="152">
       <c r="A152" s="4" t="inlineStr">
         <is>
-          <t>isBranchStockable</t>
+          <t>warehouseStatusId</t>
         </is>
       </c>
       <c r="B152" s="4" t="inlineStr">
@@ -24583,7 +24591,7 @@
       </c>
       <c r="E152" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Warehouses.isBranchStockable?</t>
+          <t>What confirmed CoCre8/SAP source should populate Warehouses.warehouseStatusId?</t>
         </is>
       </c>
       <c r="F152" s="4" t="inlineStr">
@@ -24600,12 +24608,12 @@
     <row r="153">
       <c r="A153" s="4" t="inlineStr">
         <is>
-          <t>isRemote</t>
+          <t>inventoryType</t>
         </is>
       </c>
       <c r="B153" s="4" t="inlineStr">
         <is>
-          <t>Warehouses</t>
+          <t>WarehouseStockOnHand</t>
         </is>
       </c>
       <c r="C153" s="4" t="inlineStr">
@@ -24620,7 +24628,7 @@
       </c>
       <c r="E153" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Warehouses.isRemote?</t>
+          <t>What confirmed CoCre8/SAP source should populate WarehouseStockOnHand.inventoryType?</t>
         </is>
       </c>
       <c r="F153" s="4" t="inlineStr">
@@ -24637,12 +24645,12 @@
     <row r="154">
       <c r="A154" s="4" t="inlineStr">
         <is>
-          <t>warehouseStatusId</t>
+          <t>quantityOutbound</t>
         </is>
       </c>
       <c r="B154" s="4" t="inlineStr">
         <is>
-          <t>Warehouses</t>
+          <t>WarehouseStockOnHand</t>
         </is>
       </c>
       <c r="C154" s="4" t="inlineStr">
@@ -24657,7 +24665,7 @@
       </c>
       <c r="E154" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Warehouses.warehouseStatusId?</t>
+          <t>What confirmed CoCre8/SAP source should populate WarehouseStockOnHand.quantityOutbound?</t>
         </is>
       </c>
       <c r="F154" s="4" t="inlineStr">
@@ -24674,12 +24682,12 @@
     <row r="155">
       <c r="A155" s="4" t="inlineStr">
         <is>
-          <t>inventoryType</t>
+          <t>personId</t>
         </is>
       </c>
       <c r="B155" s="4" t="inlineStr">
         <is>
-          <t>WarehouseStockOnHand</t>
+          <t>Employees</t>
         </is>
       </c>
       <c r="C155" s="4" t="inlineStr">
@@ -24694,7 +24702,7 @@
       </c>
       <c r="E155" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate WarehouseStockOnHand.inventoryType?</t>
+          <t>What confirmed CoCre8/SAP source should populate Employees.personId?</t>
         </is>
       </c>
       <c r="F155" s="4" t="inlineStr">
@@ -24711,12 +24719,12 @@
     <row r="156">
       <c r="A156" s="4" t="inlineStr">
         <is>
-          <t>quantityOutbound</t>
+          <t>role</t>
         </is>
       </c>
       <c r="B156" s="4" t="inlineStr">
         <is>
-          <t>WarehouseStockOnHand</t>
+          <t>Employees</t>
         </is>
       </c>
       <c r="C156" s="4" t="inlineStr">
@@ -24731,7 +24739,7 @@
       </c>
       <c r="E156" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate WarehouseStockOnHand.quantityOutbound?</t>
+          <t>What confirmed CoCre8/SAP source should populate Employees.role?</t>
         </is>
       </c>
       <c r="F156" s="4" t="inlineStr">
@@ -24748,7 +24756,7 @@
     <row r="157">
       <c r="A157" s="4" t="inlineStr">
         <is>
-          <t>personId</t>
+          <t>actionGroupId</t>
         </is>
       </c>
       <c r="B157" s="4" t="inlineStr">
@@ -24768,7 +24776,7 @@
       </c>
       <c r="E157" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Employees.personId?</t>
+          <t>What confirmed CoCre8/SAP source should populate Employees.actionGroupId?</t>
         </is>
       </c>
       <c r="F157" s="4" t="inlineStr">
@@ -24785,7 +24793,7 @@
     <row r="158">
       <c r="A158" s="4" t="inlineStr">
         <is>
-          <t>role</t>
+          <t>addressId</t>
         </is>
       </c>
       <c r="B158" s="4" t="inlineStr">
@@ -24805,7 +24813,7 @@
       </c>
       <c r="E158" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Employees.role?</t>
+          <t>What confirmed CoCre8/SAP source should populate Employees.addressId?</t>
         </is>
       </c>
       <c r="F158" s="4" t="inlineStr">
@@ -24822,7 +24830,7 @@
     <row r="159">
       <c r="A159" s="4" t="inlineStr">
         <is>
-          <t>actionGroupId</t>
+          <t>nodeId</t>
         </is>
       </c>
       <c r="B159" s="4" t="inlineStr">
@@ -24842,7 +24850,7 @@
       </c>
       <c r="E159" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Employees.actionGroupId?</t>
+          <t>What confirmed CoCre8/SAP source should populate Employees.nodeId?</t>
         </is>
       </c>
       <c r="F159" s="4" t="inlineStr">
@@ -24859,7 +24867,7 @@
     <row r="160">
       <c r="A160" s="4" t="inlineStr">
         <is>
-          <t>addressId</t>
+          <t>firstName</t>
         </is>
       </c>
       <c r="B160" s="4" t="inlineStr">
@@ -24879,7 +24887,7 @@
       </c>
       <c r="E160" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Employees.addressId?</t>
+          <t>What confirmed CoCre8/SAP source should populate Employees.firstName?</t>
         </is>
       </c>
       <c r="F160" s="4" t="inlineStr">
@@ -24896,7 +24904,7 @@
     <row r="161">
       <c r="A161" s="4" t="inlineStr">
         <is>
-          <t>nodeId</t>
+          <t>middleName</t>
         </is>
       </c>
       <c r="B161" s="4" t="inlineStr">
@@ -24916,7 +24924,7 @@
       </c>
       <c r="E161" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Employees.nodeId?</t>
+          <t>What confirmed CoCre8/SAP source should populate Employees.middleName?</t>
         </is>
       </c>
       <c r="F161" s="4" t="inlineStr">
@@ -24933,7 +24941,7 @@
     <row r="162">
       <c r="A162" s="4" t="inlineStr">
         <is>
-          <t>firstName</t>
+          <t>surname</t>
         </is>
       </c>
       <c r="B162" s="4" t="inlineStr">
@@ -24953,7 +24961,7 @@
       </c>
       <c r="E162" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Employees.firstName?</t>
+          <t>What confirmed CoCre8/SAP source should populate Employees.surname?</t>
         </is>
       </c>
       <c r="F162" s="4" t="inlineStr">
@@ -24970,7 +24978,7 @@
     <row r="163">
       <c r="A163" s="4" t="inlineStr">
         <is>
-          <t>middleName</t>
+          <t>isActive</t>
         </is>
       </c>
       <c r="B163" s="4" t="inlineStr">
@@ -24990,7 +24998,7 @@
       </c>
       <c r="E163" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Employees.middleName?</t>
+          <t>What confirmed CoCre8/SAP source should populate Employees.isActive?</t>
         </is>
       </c>
       <c r="F163" s="4" t="inlineStr">
@@ -25007,7 +25015,7 @@
     <row r="164">
       <c r="A164" s="4" t="inlineStr">
         <is>
-          <t>surname</t>
+          <t>telephoneNumber</t>
         </is>
       </c>
       <c r="B164" s="4" t="inlineStr">
@@ -25027,7 +25035,7 @@
       </c>
       <c r="E164" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Employees.surname?</t>
+          <t>What confirmed CoCre8/SAP source should populate Employees.telephoneNumber?</t>
         </is>
       </c>
       <c r="F164" s="4" t="inlineStr">
@@ -25044,12 +25052,12 @@
     <row r="165">
       <c r="A165" s="4" t="inlineStr">
         <is>
-          <t>isActive</t>
+          <t>orderNumber</t>
         </is>
       </c>
       <c r="B165" s="4" t="inlineStr">
         <is>
-          <t>Employees</t>
+          <t>PartsUsage</t>
         </is>
       </c>
       <c r="C165" s="4" t="inlineStr">
@@ -25064,7 +25072,7 @@
       </c>
       <c r="E165" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Employees.isActive?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartsUsage.orderNumber?</t>
         </is>
       </c>
       <c r="F165" s="4" t="inlineStr">
@@ -25081,12 +25089,12 @@
     <row r="166">
       <c r="A166" s="4" t="inlineStr">
         <is>
-          <t>telephoneNumber</t>
+          <t>requestId</t>
         </is>
       </c>
       <c r="B166" s="4" t="inlineStr">
         <is>
-          <t>Employees</t>
+          <t>PartsUsage</t>
         </is>
       </c>
       <c r="C166" s="4" t="inlineStr">
@@ -25101,7 +25109,7 @@
       </c>
       <c r="E166" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Employees.telephoneNumber?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartsUsage.requestId?</t>
         </is>
       </c>
       <c r="F166" s="4" t="inlineStr">
@@ -25118,7 +25126,7 @@
     <row r="167">
       <c r="A167" s="4" t="inlineStr">
         <is>
-          <t>orderNumber</t>
+          <t>customerCompanyCode</t>
         </is>
       </c>
       <c r="B167" s="4" t="inlineStr">
@@ -25138,7 +25146,7 @@
       </c>
       <c r="E167" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartsUsage.orderNumber?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartsUsage.customerCompanyCode?</t>
         </is>
       </c>
       <c r="F167" s="4" t="inlineStr">
@@ -25155,7 +25163,7 @@
     <row r="168">
       <c r="A168" s="4" t="inlineStr">
         <is>
-          <t>requestId</t>
+          <t>orderType</t>
         </is>
       </c>
       <c r="B168" s="4" t="inlineStr">
@@ -25175,7 +25183,7 @@
       </c>
       <c r="E168" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartsUsage.requestId?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartsUsage.orderType?</t>
         </is>
       </c>
       <c r="F168" s="4" t="inlineStr">
@@ -25192,7 +25200,7 @@
     <row r="169">
       <c r="A169" s="4" t="inlineStr">
         <is>
-          <t>customerCompanyCode</t>
+          <t>orderStatus</t>
         </is>
       </c>
       <c r="B169" s="4" t="inlineStr">
@@ -25212,7 +25220,7 @@
       </c>
       <c r="E169" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartsUsage.customerCompanyCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartsUsage.orderStatus?</t>
         </is>
       </c>
       <c r="F169" s="4" t="inlineStr">
@@ -25229,7 +25237,7 @@
     <row r="170">
       <c r="A170" s="4" t="inlineStr">
         <is>
-          <t>orderType</t>
+          <t>orderStartDatetime</t>
         </is>
       </c>
       <c r="B170" s="4" t="inlineStr">
@@ -25249,7 +25257,7 @@
       </c>
       <c r="E170" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartsUsage.orderType?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartsUsage.orderStartDatetime?</t>
         </is>
       </c>
       <c r="F170" s="4" t="inlineStr">
@@ -25266,7 +25274,7 @@
     <row r="171">
       <c r="A171" s="4" t="inlineStr">
         <is>
-          <t>orderStatus</t>
+          <t>requestTicketDateTime</t>
         </is>
       </c>
       <c r="B171" s="4" t="inlineStr">
@@ -25286,7 +25294,7 @@
       </c>
       <c r="E171" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartsUsage.orderStatus?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartsUsage.requestTicketDateTime?</t>
         </is>
       </c>
       <c r="F171" s="4" t="inlineStr">
@@ -25303,7 +25311,7 @@
     <row r="172">
       <c r="A172" s="4" t="inlineStr">
         <is>
-          <t>orderStartDatetime</t>
+          <t>siteCompanyCode</t>
         </is>
       </c>
       <c r="B172" s="4" t="inlineStr">
@@ -25323,7 +25331,7 @@
       </c>
       <c r="E172" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartsUsage.orderStartDatetime?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartsUsage.siteCompanyCode?</t>
         </is>
       </c>
       <c r="F172" s="4" t="inlineStr">
@@ -25340,7 +25348,7 @@
     <row r="173">
       <c r="A173" s="4" t="inlineStr">
         <is>
-          <t>requestTicketDateTime</t>
+          <t>partCode</t>
         </is>
       </c>
       <c r="B173" s="4" t="inlineStr">
@@ -25360,7 +25368,7 @@
       </c>
       <c r="E173" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartsUsage.requestTicketDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartsUsage.partCode?</t>
         </is>
       </c>
       <c r="F173" s="4" t="inlineStr">
@@ -25377,7 +25385,7 @@
     <row r="174">
       <c r="A174" s="4" t="inlineStr">
         <is>
-          <t>siteCompanyCode</t>
+          <t>Warehouse</t>
         </is>
       </c>
       <c r="B174" s="4" t="inlineStr">
@@ -25397,7 +25405,7 @@
       </c>
       <c r="E174" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartsUsage.siteCompanyCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartsUsage.Warehouse?</t>
         </is>
       </c>
       <c r="F174" s="4" t="inlineStr">
@@ -25414,7 +25422,7 @@
     <row r="175">
       <c r="A175" s="4" t="inlineStr">
         <is>
-          <t>partCode</t>
+          <t>assignedPersonCode</t>
         </is>
       </c>
       <c r="B175" s="4" t="inlineStr">
@@ -25434,7 +25442,7 @@
       </c>
       <c r="E175" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartsUsage.partCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartsUsage.assignedPersonCode?</t>
         </is>
       </c>
       <c r="F175" s="4" t="inlineStr">
@@ -25451,7 +25459,7 @@
     <row r="176">
       <c r="A176" s="4" t="inlineStr">
         <is>
-          <t>Warehouse</t>
+          <t>resolvedDateTime</t>
         </is>
       </c>
       <c r="B176" s="4" t="inlineStr">
@@ -25471,7 +25479,7 @@
       </c>
       <c r="E176" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartsUsage.Warehouse?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartsUsage.resolvedDateTime?</t>
         </is>
       </c>
       <c r="F176" s="4" t="inlineStr">
@@ -25488,7 +25496,7 @@
     <row r="177">
       <c r="A177" s="4" t="inlineStr">
         <is>
-          <t>assignedPersonCode</t>
+          <t>serialNumber</t>
         </is>
       </c>
       <c r="B177" s="4" t="inlineStr">
@@ -25508,7 +25516,7 @@
       </c>
       <c r="E177" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartsUsage.assignedPersonCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartsUsage.serialNumber?</t>
         </is>
       </c>
       <c r="F177" s="4" t="inlineStr">
@@ -25525,7 +25533,7 @@
     <row r="178">
       <c r="A178" s="4" t="inlineStr">
         <is>
-          <t>resolvedDateTime</t>
+          <t>quantityUsed</t>
         </is>
       </c>
       <c r="B178" s="4" t="inlineStr">
@@ -25545,7 +25553,7 @@
       </c>
       <c r="E178" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartsUsage.resolvedDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartsUsage.quantityUsed?</t>
         </is>
       </c>
       <c r="F178" s="4" t="inlineStr">
@@ -25562,7 +25570,7 @@
     <row r="179">
       <c r="A179" s="4" t="inlineStr">
         <is>
-          <t>serialNumber</t>
+          <t>relCompanyId</t>
         </is>
       </c>
       <c r="B179" s="4" t="inlineStr">
@@ -25582,7 +25590,7 @@
       </c>
       <c r="E179" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartsUsage.serialNumber?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartsUsage.relCompanyId?</t>
         </is>
       </c>
       <c r="F179" s="4" t="inlineStr">
@@ -25599,7 +25607,7 @@
     <row r="180">
       <c r="A180" s="4" t="inlineStr">
         <is>
-          <t>quantityUsed</t>
+          <t>partsUsedDateTime</t>
         </is>
       </c>
       <c r="B180" s="4" t="inlineStr">
@@ -25619,7 +25627,7 @@
       </c>
       <c r="E180" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartsUsage.quantityUsed?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartsUsage.partsUsedDateTime?</t>
         </is>
       </c>
       <c r="F180" s="4" t="inlineStr">
@@ -25636,7 +25644,7 @@
     <row r="181">
       <c r="A181" s="4" t="inlineStr">
         <is>
-          <t>relCompanyId</t>
+          <t>deviceSerialNumber</t>
         </is>
       </c>
       <c r="B181" s="4" t="inlineStr">
@@ -25656,7 +25664,7 @@
       </c>
       <c r="E181" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartsUsage.relCompanyId?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartsUsage.deviceSerialNumber?</t>
         </is>
       </c>
       <c r="F181" s="4" t="inlineStr">
@@ -25673,12 +25681,12 @@
     <row r="182">
       <c r="A182" s="4" t="inlineStr">
         <is>
-          <t>partsUsedDateTime</t>
+          <t>orderNumber</t>
         </is>
       </c>
       <c r="B182" s="4" t="inlineStr">
         <is>
-          <t>PartsUsage</t>
+          <t>ServiceOrder</t>
         </is>
       </c>
       <c r="C182" s="4" t="inlineStr">
@@ -25693,7 +25701,7 @@
       </c>
       <c r="E182" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartsUsage.partsUsedDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.orderNumber?</t>
         </is>
       </c>
       <c r="F182" s="4" t="inlineStr">
@@ -25710,12 +25718,12 @@
     <row r="183">
       <c r="A183" s="4" t="inlineStr">
         <is>
-          <t>deviceSerialNumber</t>
+          <t>location</t>
         </is>
       </c>
       <c r="B183" s="4" t="inlineStr">
         <is>
-          <t>PartsUsage</t>
+          <t>ServiceOrder</t>
         </is>
       </c>
       <c r="C183" s="4" t="inlineStr">
@@ -25730,7 +25738,7 @@
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartsUsage.deviceSerialNumber?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.location?</t>
         </is>
       </c>
       <c r="F183" s="4" t="inlineStr">
@@ -25747,7 +25755,7 @@
     <row r="184">
       <c r="A184" s="4" t="inlineStr">
         <is>
-          <t>orderNumber</t>
+          <t>eta</t>
         </is>
       </c>
       <c r="B184" s="4" t="inlineStr">
@@ -25767,7 +25775,7 @@
       </c>
       <c r="E184" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.orderNumber?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.eta?</t>
         </is>
       </c>
       <c r="F184" s="4" t="inlineStr">
@@ -25784,7 +25792,7 @@
     <row r="185">
       <c r="A185" s="4" t="inlineStr">
         <is>
-          <t>location</t>
+          <t>actualEta</t>
         </is>
       </c>
       <c r="B185" s="4" t="inlineStr">
@@ -25804,7 +25812,7 @@
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.location?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.actualEta?</t>
         </is>
       </c>
       <c r="F185" s="4" t="inlineStr">
@@ -25821,7 +25829,7 @@
     <row r="186">
       <c r="A186" s="4" t="inlineStr">
         <is>
-          <t>eta</t>
+          <t>actualResolveDateTime</t>
         </is>
       </c>
       <c r="B186" s="4" t="inlineStr">
@@ -25841,7 +25849,7 @@
       </c>
       <c r="E186" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.eta?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.actualResolveDateTime?</t>
         </is>
       </c>
       <c r="F186" s="4" t="inlineStr">
@@ -25858,7 +25866,7 @@
     <row r="187">
       <c r="A187" s="4" t="inlineStr">
         <is>
-          <t>actualEta</t>
+          <t>recallDateTime</t>
         </is>
       </c>
       <c r="B187" s="4" t="inlineStr">
@@ -25878,7 +25886,7 @@
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.actualEta?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.recallDateTime?</t>
         </is>
       </c>
       <c r="F187" s="4" t="inlineStr">
@@ -25895,7 +25903,7 @@
     <row r="188">
       <c r="A188" s="4" t="inlineStr">
         <is>
-          <t>actualResolveDateTime</t>
+          <t>actualRecallDateTime</t>
         </is>
       </c>
       <c r="B188" s="4" t="inlineStr">
@@ -25915,7 +25923,7 @@
       </c>
       <c r="E188" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.actualResolveDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.actualRecallDateTime?</t>
         </is>
       </c>
       <c r="F188" s="4" t="inlineStr">
@@ -25932,7 +25940,7 @@
     <row r="189">
       <c r="A189" s="4" t="inlineStr">
         <is>
-          <t>recallDateTime</t>
+          <t>slaEtaClock</t>
         </is>
       </c>
       <c r="B189" s="4" t="inlineStr">
@@ -25952,7 +25960,7 @@
       </c>
       <c r="E189" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.recallDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaEtaClock?</t>
         </is>
       </c>
       <c r="F189" s="4" t="inlineStr">
@@ -25969,7 +25977,7 @@
     <row r="190">
       <c r="A190" s="4" t="inlineStr">
         <is>
-          <t>actualRecallDateTime</t>
+          <t>slaResolveClock</t>
         </is>
       </c>
       <c r="B190" s="4" t="inlineStr">
@@ -25989,7 +25997,7 @@
       </c>
       <c r="E190" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.actualRecallDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaResolveClock?</t>
         </is>
       </c>
       <c r="F190" s="4" t="inlineStr">
@@ -26006,7 +26014,7 @@
     <row r="191">
       <c r="A191" s="4" t="inlineStr">
         <is>
-          <t>slaEtaClock</t>
+          <t>slaFailureCode</t>
         </is>
       </c>
       <c r="B191" s="4" t="inlineStr">
@@ -26026,7 +26034,7 @@
       </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaEtaClock?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaFailureCode?</t>
         </is>
       </c>
       <c r="F191" s="4" t="inlineStr">
@@ -26043,7 +26051,7 @@
     <row r="192">
       <c r="A192" s="4" t="inlineStr">
         <is>
-          <t>slaResolveClock</t>
+          <t>slaEtaHit</t>
         </is>
       </c>
       <c r="B192" s="4" t="inlineStr">
@@ -26063,7 +26071,7 @@
       </c>
       <c r="E192" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaResolveClock?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaEtaHit?</t>
         </is>
       </c>
       <c r="F192" s="4" t="inlineStr">
@@ -26080,7 +26088,7 @@
     <row r="193">
       <c r="A193" s="4" t="inlineStr">
         <is>
-          <t>slaFailureCode</t>
+          <t>slaResolvedDateTime</t>
         </is>
       </c>
       <c r="B193" s="4" t="inlineStr">
@@ -26100,7 +26108,7 @@
       </c>
       <c r="E193" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaFailureCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaResolvedDateTime?</t>
         </is>
       </c>
       <c r="F193" s="4" t="inlineStr">
@@ -26117,12 +26125,12 @@
     <row r="194">
       <c r="A194" s="4" t="inlineStr">
         <is>
-          <t>slaEtaHit</t>
+          <t>orderNumber</t>
         </is>
       </c>
       <c r="B194" s="4" t="inlineStr">
         <is>
-          <t>ServiceOrder</t>
+          <t>RepairOrder</t>
         </is>
       </c>
       <c r="C194" s="4" t="inlineStr">
@@ -26137,7 +26145,7 @@
       </c>
       <c r="E194" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaEtaHit?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.orderNumber?</t>
         </is>
       </c>
       <c r="F194" s="4" t="inlineStr">
@@ -26154,12 +26162,12 @@
     <row r="195">
       <c r="A195" s="4" t="inlineStr">
         <is>
-          <t>slaResolvedDateTime</t>
+          <t>requestId</t>
         </is>
       </c>
       <c r="B195" s="4" t="inlineStr">
         <is>
-          <t>ServiceOrder</t>
+          <t>RepairOrder</t>
         </is>
       </c>
       <c r="C195" s="4" t="inlineStr">
@@ -26174,7 +26182,7 @@
       </c>
       <c r="E195" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ServiceOrder.slaResolvedDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.requestId?</t>
         </is>
       </c>
       <c r="F195" s="4" t="inlineStr">
@@ -26191,7 +26199,7 @@
     <row r="196">
       <c r="A196" s="4" t="inlineStr">
         <is>
-          <t>orderNumber</t>
+          <t>customerCompanyCode</t>
         </is>
       </c>
       <c r="B196" s="4" t="inlineStr">
@@ -26211,7 +26219,7 @@
       </c>
       <c r="E196" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.orderNumber?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.customerCompanyCode?</t>
         </is>
       </c>
       <c r="F196" s="4" t="inlineStr">
@@ -26228,7 +26236,7 @@
     <row r="197">
       <c r="A197" s="4" t="inlineStr">
         <is>
-          <t>requestId</t>
+          <t>orderStatus</t>
         </is>
       </c>
       <c r="B197" s="4" t="inlineStr">
@@ -26248,7 +26256,7 @@
       </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.requestId?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.orderStatus?</t>
         </is>
       </c>
       <c r="F197" s="4" t="inlineStr">
@@ -26265,7 +26273,7 @@
     <row r="198">
       <c r="A198" s="4" t="inlineStr">
         <is>
-          <t>customerCompanyCode</t>
+          <t>orderStartDatetime</t>
         </is>
       </c>
       <c r="B198" s="4" t="inlineStr">
@@ -26285,7 +26293,7 @@
       </c>
       <c r="E198" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.customerCompanyCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.orderStartDatetime?</t>
         </is>
       </c>
       <c r="F198" s="4" t="inlineStr">
@@ -26302,7 +26310,7 @@
     <row r="199">
       <c r="A199" s="4" t="inlineStr">
         <is>
-          <t>orderStatus</t>
+          <t>siteCompanyCode</t>
         </is>
       </c>
       <c r="B199" s="4" t="inlineStr">
@@ -26322,7 +26330,7 @@
       </c>
       <c r="E199" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.orderStatus?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.siteCompanyCode?</t>
         </is>
       </c>
       <c r="F199" s="4" t="inlineStr">
@@ -26339,7 +26347,7 @@
     <row r="200">
       <c r="A200" s="4" t="inlineStr">
         <is>
-          <t>orderStartDatetime</t>
+          <t>repairType</t>
         </is>
       </c>
       <c r="B200" s="4" t="inlineStr">
@@ -26359,7 +26367,7 @@
       </c>
       <c r="E200" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.orderStartDatetime?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.repairType?</t>
         </is>
       </c>
       <c r="F200" s="4" t="inlineStr">
@@ -26376,7 +26384,7 @@
     <row r="201">
       <c r="A201" s="4" t="inlineStr">
         <is>
-          <t>siteCompanyCode</t>
+          <t>partsOrderDateTime</t>
         </is>
       </c>
       <c r="B201" s="4" t="inlineStr">
@@ -26396,7 +26404,7 @@
       </c>
       <c r="E201" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.siteCompanyCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.partsOrderDateTime?</t>
         </is>
       </c>
       <c r="F201" s="4" t="inlineStr">
@@ -26413,7 +26421,7 @@
     <row r="202">
       <c r="A202" s="4" t="inlineStr">
         <is>
-          <t>repairType</t>
+          <t>partsReceivedDateTime</t>
         </is>
       </c>
       <c r="B202" s="4" t="inlineStr">
@@ -26433,7 +26441,7 @@
       </c>
       <c r="E202" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.repairType?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.partsReceivedDateTime?</t>
         </is>
       </c>
       <c r="F202" s="4" t="inlineStr">
@@ -26450,7 +26458,7 @@
     <row r="203">
       <c r="A203" s="4" t="inlineStr">
         <is>
-          <t>partsOrderDateTime</t>
+          <t>repairCode</t>
         </is>
       </c>
       <c r="B203" s="4" t="inlineStr">
@@ -26470,7 +26478,7 @@
       </c>
       <c r="E203" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.partsOrderDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.repairCode?</t>
         </is>
       </c>
       <c r="F203" s="4" t="inlineStr">
@@ -26487,7 +26495,7 @@
     <row r="204">
       <c r="A204" s="4" t="inlineStr">
         <is>
-          <t>partsReceivedDateTime</t>
+          <t>repairCompany</t>
         </is>
       </c>
       <c r="B204" s="4" t="inlineStr">
@@ -26507,7 +26515,7 @@
       </c>
       <c r="E204" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.partsReceivedDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.repairCompany?</t>
         </is>
       </c>
       <c r="F204" s="4" t="inlineStr">
@@ -26524,7 +26532,7 @@
     <row r="205">
       <c r="A205" s="4" t="inlineStr">
         <is>
-          <t>repairCode</t>
+          <t>raStatus</t>
         </is>
       </c>
       <c r="B205" s="4" t="inlineStr">
@@ -26544,7 +26552,7 @@
       </c>
       <c r="E205" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.repairCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.raStatus?</t>
         </is>
       </c>
       <c r="F205" s="4" t="inlineStr">
@@ -26561,7 +26569,7 @@
     <row r="206">
       <c r="A206" s="4" t="inlineStr">
         <is>
-          <t>repairCompany</t>
+          <t>Warehouse</t>
         </is>
       </c>
       <c r="B206" s="4" t="inlineStr">
@@ -26581,7 +26589,7 @@
       </c>
       <c r="E206" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.repairCompany?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.Warehouse?</t>
         </is>
       </c>
       <c r="F206" s="4" t="inlineStr">
@@ -26598,7 +26606,7 @@
     <row r="207">
       <c r="A207" s="4" t="inlineStr">
         <is>
-          <t>raStatus</t>
+          <t>assignedPerson</t>
         </is>
       </c>
       <c r="B207" s="4" t="inlineStr">
@@ -26618,7 +26626,7 @@
       </c>
       <c r="E207" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.raStatus?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.assignedPerson?</t>
         </is>
       </c>
       <c r="F207" s="4" t="inlineStr">
@@ -26635,7 +26643,7 @@
     <row r="208">
       <c r="A208" s="4" t="inlineStr">
         <is>
-          <t>Warehouse</t>
+          <t>orderedPartId</t>
         </is>
       </c>
       <c r="B208" s="4" t="inlineStr">
@@ -26655,7 +26663,7 @@
       </c>
       <c r="E208" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.Warehouse?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.orderedPartId?</t>
         </is>
       </c>
       <c r="F208" s="4" t="inlineStr">
@@ -26672,7 +26680,7 @@
     <row r="209">
       <c r="A209" s="4" t="inlineStr">
         <is>
-          <t>assignedPerson</t>
+          <t>actualPartId</t>
         </is>
       </c>
       <c r="B209" s="4" t="inlineStr">
@@ -26692,7 +26700,7 @@
       </c>
       <c r="E209" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.assignedPerson?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.actualPartId?</t>
         </is>
       </c>
       <c r="F209" s="4" t="inlineStr">
@@ -26709,7 +26717,7 @@
     <row r="210">
       <c r="A210" s="4" t="inlineStr">
         <is>
-          <t>orderedPartId</t>
+          <t>resolvedDateTime</t>
         </is>
       </c>
       <c r="B210" s="4" t="inlineStr">
@@ -26729,7 +26737,7 @@
       </c>
       <c r="E210" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.orderedPartId?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.resolvedDateTime?</t>
         </is>
       </c>
       <c r="F210" s="4" t="inlineStr">
@@ -26746,7 +26754,7 @@
     <row r="211">
       <c r="A211" s="4" t="inlineStr">
         <is>
-          <t>actualPartId</t>
+          <t>serialNumber</t>
         </is>
       </c>
       <c r="B211" s="4" t="inlineStr">
@@ -26766,7 +26774,7 @@
       </c>
       <c r="E211" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.actualPartId?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.serialNumber?</t>
         </is>
       </c>
       <c r="F211" s="4" t="inlineStr">
@@ -26783,7 +26791,7 @@
     <row r="212">
       <c r="A212" s="4" t="inlineStr">
         <is>
-          <t>resolvedDateTime</t>
+          <t>quantityUsed</t>
         </is>
       </c>
       <c r="B212" s="4" t="inlineStr">
@@ -26803,7 +26811,7 @@
       </c>
       <c r="E212" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.resolvedDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.quantityUsed?</t>
         </is>
       </c>
       <c r="F212" s="4" t="inlineStr">
@@ -26820,7 +26828,7 @@
     <row r="213">
       <c r="A213" s="4" t="inlineStr">
         <is>
-          <t>serialNumber</t>
+          <t>relCompanyId</t>
         </is>
       </c>
       <c r="B213" s="4" t="inlineStr">
@@ -26840,7 +26848,7 @@
       </c>
       <c r="E213" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.serialNumber?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.relCompanyId?</t>
         </is>
       </c>
       <c r="F213" s="4" t="inlineStr">
@@ -26857,7 +26865,7 @@
     <row r="214">
       <c r="A214" s="4" t="inlineStr">
         <is>
-          <t>quantityUsed</t>
+          <t>partsUsedDateTime</t>
         </is>
       </c>
       <c r="B214" s="4" t="inlineStr">
@@ -26877,7 +26885,7 @@
       </c>
       <c r="E214" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.quantityUsed?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.partsUsedDateTime?</t>
         </is>
       </c>
       <c r="F214" s="4" t="inlineStr">
@@ -26894,7 +26902,7 @@
     <row r="215">
       <c r="A215" s="4" t="inlineStr">
         <is>
-          <t>relCompanyId</t>
+          <t>deviceSerialNumber</t>
         </is>
       </c>
       <c r="B215" s="4" t="inlineStr">
@@ -26914,7 +26922,7 @@
       </c>
       <c r="E215" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.relCompanyId?</t>
+          <t>What confirmed CoCre8/SAP source should populate RepairOrder.deviceSerialNumber?</t>
         </is>
       </c>
       <c r="F215" s="4" t="inlineStr">
@@ -26931,12 +26939,12 @@
     <row r="216">
       <c r="A216" s="4" t="inlineStr">
         <is>
-          <t>partsUsedDateTime</t>
+          <t>partCode</t>
         </is>
       </c>
       <c r="B216" s="4" t="inlineStr">
         <is>
-          <t>RepairOrder</t>
+          <t>PartCost</t>
         </is>
       </c>
       <c r="C216" s="4" t="inlineStr">
@@ -26951,7 +26959,7 @@
       </c>
       <c r="E216" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.partsUsedDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartCost.partCode?</t>
         </is>
       </c>
       <c r="F216" s="4" t="inlineStr">
@@ -26968,12 +26976,12 @@
     <row r="217">
       <c r="A217" s="4" t="inlineStr">
         <is>
-          <t>deviceSerialNumber</t>
+          <t>cost</t>
         </is>
       </c>
       <c r="B217" s="4" t="inlineStr">
         <is>
-          <t>RepairOrder</t>
+          <t>PartCost</t>
         </is>
       </c>
       <c r="C217" s="4" t="inlineStr">
@@ -26988,7 +26996,7 @@
       </c>
       <c r="E217" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate RepairOrder.deviceSerialNumber?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartCost.cost?</t>
         </is>
       </c>
       <c r="F217" s="4" t="inlineStr">
@@ -27005,7 +27013,7 @@
     <row r="218">
       <c r="A218" s="4" t="inlineStr">
         <is>
-          <t>partCode</t>
+          <t>currencyCode</t>
         </is>
       </c>
       <c r="B218" s="4" t="inlineStr">
@@ -27025,7 +27033,7 @@
       </c>
       <c r="E218" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartCost.partCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartCost.currencyCode?</t>
         </is>
       </c>
       <c r="F218" s="4" t="inlineStr">
@@ -27042,7 +27050,7 @@
     <row r="219">
       <c r="A219" s="4" t="inlineStr">
         <is>
-          <t>cost</t>
+          <t>averageCost</t>
         </is>
       </c>
       <c r="B219" s="4" t="inlineStr">
@@ -27062,7 +27070,7 @@
       </c>
       <c r="E219" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartCost.cost?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartCost.averageCost?</t>
         </is>
       </c>
       <c r="F219" s="4" t="inlineStr">
@@ -27079,7 +27087,7 @@
     <row r="220">
       <c r="A220" s="4" t="inlineStr">
         <is>
-          <t>currencyCode</t>
+          <t>averageRepairCost</t>
         </is>
       </c>
       <c r="B220" s="4" t="inlineStr">
@@ -27099,7 +27107,7 @@
       </c>
       <c r="E220" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartCost.currencyCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartCost.averageRepairCost?</t>
         </is>
       </c>
       <c r="F220" s="4" t="inlineStr">
@@ -27116,12 +27124,12 @@
     <row r="221">
       <c r="A221" s="4" t="inlineStr">
         <is>
-          <t>averageCost</t>
+          <t>partCode</t>
         </is>
       </c>
       <c r="B221" s="4" t="inlineStr">
         <is>
-          <t>PartCost</t>
+          <t>Models</t>
         </is>
       </c>
       <c r="C221" s="4" t="inlineStr">
@@ -27136,7 +27144,7 @@
       </c>
       <c r="E221" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartCost.averageCost?</t>
+          <t>What confirmed CoCre8/SAP source should populate Models.partCode?</t>
         </is>
       </c>
       <c r="F221" s="4" t="inlineStr">
@@ -27153,12 +27161,12 @@
     <row r="222">
       <c r="A222" s="4" t="inlineStr">
         <is>
-          <t>averageRepairCost</t>
+          <t>modelCode</t>
         </is>
       </c>
       <c r="B222" s="4" t="inlineStr">
         <is>
-          <t>PartCost</t>
+          <t>Models</t>
         </is>
       </c>
       <c r="C222" s="4" t="inlineStr">
@@ -27173,7 +27181,7 @@
       </c>
       <c r="E222" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartCost.averageRepairCost?</t>
+          <t>What confirmed CoCre8/SAP source should populate Models.modelCode?</t>
         </is>
       </c>
       <c r="F222" s="4" t="inlineStr">
@@ -27190,7 +27198,7 @@
     <row r="223">
       <c r="A223" s="4" t="inlineStr">
         <is>
-          <t>partCode</t>
+          <t>modelDescription</t>
         </is>
       </c>
       <c r="B223" s="4" t="inlineStr">
@@ -27210,7 +27218,7 @@
       </c>
       <c r="E223" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Models.partCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate Models.modelDescription?</t>
         </is>
       </c>
       <c r="F223" s="4" t="inlineStr">
@@ -27227,12 +27235,12 @@
     <row r="224">
       <c r="A224" s="4" t="inlineStr">
         <is>
-          <t>modelCode</t>
+          <t>inventoryTransferImoId</t>
         </is>
       </c>
       <c r="B224" s="4" t="inlineStr">
         <is>
-          <t>Models</t>
+          <t>InventoryTransfers</t>
         </is>
       </c>
       <c r="C224" s="4" t="inlineStr">
@@ -27247,7 +27255,7 @@
       </c>
       <c r="E224" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Models.modelCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.inventoryTransferImoId?</t>
         </is>
       </c>
       <c r="F224" s="4" t="inlineStr">
@@ -27264,12 +27272,12 @@
     <row r="225">
       <c r="A225" s="4" t="inlineStr">
         <is>
-          <t>modelDescription</t>
+          <t>createdDateTime</t>
         </is>
       </c>
       <c r="B225" s="4" t="inlineStr">
         <is>
-          <t>Models</t>
+          <t>InventoryTransfers</t>
         </is>
       </c>
       <c r="C225" s="4" t="inlineStr">
@@ -27284,7 +27292,7 @@
       </c>
       <c r="E225" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Models.modelDescription?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.createdDateTime?</t>
         </is>
       </c>
       <c r="F225" s="4" t="inlineStr">
@@ -27301,7 +27309,7 @@
     <row r="226">
       <c r="A226" s="4" t="inlineStr">
         <is>
-          <t>inventoryTransferImoId</t>
+          <t>completedDateTime</t>
         </is>
       </c>
       <c r="B226" s="4" t="inlineStr">
@@ -27321,7 +27329,7 @@
       </c>
       <c r="E226" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.inventoryTransferImoId?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.completedDateTime?</t>
         </is>
       </c>
       <c r="F226" s="4" t="inlineStr">
@@ -27338,7 +27346,7 @@
     <row r="227">
       <c r="A227" s="4" t="inlineStr">
         <is>
-          <t>createdDateTime</t>
+          <t>fromWarehouseId</t>
         </is>
       </c>
       <c r="B227" s="4" t="inlineStr">
@@ -27358,7 +27366,7 @@
       </c>
       <c r="E227" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.createdDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.fromWarehouseId?</t>
         </is>
       </c>
       <c r="F227" s="4" t="inlineStr">
@@ -27375,7 +27383,7 @@
     <row r="228">
       <c r="A228" s="4" t="inlineStr">
         <is>
-          <t>completedDateTime</t>
+          <t>toWarehouseId</t>
         </is>
       </c>
       <c r="B228" s="4" t="inlineStr">
@@ -27395,7 +27403,7 @@
       </c>
       <c r="E228" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.completedDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.toWarehouseId?</t>
         </is>
       </c>
       <c r="F228" s="4" t="inlineStr">
@@ -27412,7 +27420,7 @@
     <row r="229">
       <c r="A229" s="4" t="inlineStr">
         <is>
-          <t>fromWarehouseId</t>
+          <t>demandStatus</t>
         </is>
       </c>
       <c r="B229" s="4" t="inlineStr">
@@ -27432,7 +27440,7 @@
       </c>
       <c r="E229" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.fromWarehouseId?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.demandStatus?</t>
         </is>
       </c>
       <c r="F229" s="4" t="inlineStr">
@@ -27449,7 +27457,7 @@
     <row r="230">
       <c r="A230" s="4" t="inlineStr">
         <is>
-          <t>toWarehouseId</t>
+          <t>orderStatusIsClosed</t>
         </is>
       </c>
       <c r="B230" s="4" t="inlineStr">
@@ -27469,7 +27477,7 @@
       </c>
       <c r="E230" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.toWarehouseId?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.orderStatusIsClosed?</t>
         </is>
       </c>
       <c r="F230" s="4" t="inlineStr">
@@ -27486,7 +27494,7 @@
     <row r="231">
       <c r="A231" s="4" t="inlineStr">
         <is>
-          <t>demandStatus</t>
+          <t>loClass</t>
         </is>
       </c>
       <c r="B231" s="4" t="inlineStr">
@@ -27506,7 +27514,7 @@
       </c>
       <c r="E231" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.demandStatus?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.loClass?</t>
         </is>
       </c>
       <c r="F231" s="4" t="inlineStr">
@@ -27523,7 +27531,7 @@
     <row r="232">
       <c r="A232" s="4" t="inlineStr">
         <is>
-          <t>orderStatusIsClosed</t>
+          <t>movementType</t>
         </is>
       </c>
       <c r="B232" s="4" t="inlineStr">
@@ -27543,7 +27551,7 @@
       </c>
       <c r="E232" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.orderStatusIsClosed?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.movementType?</t>
         </is>
       </c>
       <c r="F232" s="4" t="inlineStr">
@@ -27560,7 +27568,7 @@
     <row r="233">
       <c r="A233" s="4" t="inlineStr">
         <is>
-          <t>loClass</t>
+          <t>addressId</t>
         </is>
       </c>
       <c r="B233" s="4" t="inlineStr">
@@ -27580,7 +27588,7 @@
       </c>
       <c r="E233" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.loClass?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.addressId?</t>
         </is>
       </c>
       <c r="F233" s="4" t="inlineStr">
@@ -27597,7 +27605,7 @@
     <row r="234">
       <c r="A234" s="4" t="inlineStr">
         <is>
-          <t>movementType</t>
+          <t>isResolved</t>
         </is>
       </c>
       <c r="B234" s="4" t="inlineStr">
@@ -27617,7 +27625,7 @@
       </c>
       <c r="E234" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.movementType?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.isResolved?</t>
         </is>
       </c>
       <c r="F234" s="4" t="inlineStr">
@@ -27634,7 +27642,7 @@
     <row r="235">
       <c r="A235" s="4" t="inlineStr">
         <is>
-          <t>addressId</t>
+          <t>partNumber</t>
         </is>
       </c>
       <c r="B235" s="4" t="inlineStr">
@@ -27654,7 +27662,7 @@
       </c>
       <c r="E235" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.addressId?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.partNumber?</t>
         </is>
       </c>
       <c r="F235" s="4" t="inlineStr">
@@ -27671,7 +27679,7 @@
     <row r="236">
       <c r="A236" s="4" t="inlineStr">
         <is>
-          <t>isResolved</t>
+          <t>quantity</t>
         </is>
       </c>
       <c r="B236" s="4" t="inlineStr">
@@ -27691,7 +27699,7 @@
       </c>
       <c r="E236" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.isResolved?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.quantity?</t>
         </is>
       </c>
       <c r="F236" s="4" t="inlineStr">
@@ -27708,7 +27716,7 @@
     <row r="237">
       <c r="A237" s="4" t="inlineStr">
         <is>
-          <t>partNumber</t>
+          <t>shipListCode</t>
         </is>
       </c>
       <c r="B237" s="4" t="inlineStr">
@@ -27728,7 +27736,7 @@
       </c>
       <c r="E237" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.partNumber?</t>
+          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.shipListCode?</t>
         </is>
       </c>
       <c r="F237" s="4" t="inlineStr">
@@ -27745,12 +27753,12 @@
     <row r="238">
       <c r="A238" s="4" t="inlineStr">
         <is>
-          <t>quantity</t>
+          <t>purchaseOrderNumber</t>
         </is>
       </c>
       <c r="B238" s="4" t="inlineStr">
         <is>
-          <t>InventoryTransfers</t>
+          <t>PurchaseOrders</t>
         </is>
       </c>
       <c r="C238" s="4" t="inlineStr">
@@ -27765,7 +27773,7 @@
       </c>
       <c r="E238" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.quantity?</t>
+          <t>What confirmed CoCre8/SAP source should populate PurchaseOrders.purchaseOrderNumber?</t>
         </is>
       </c>
       <c r="F238" s="4" t="inlineStr">
@@ -27782,12 +27790,12 @@
     <row r="239">
       <c r="A239" s="4" t="inlineStr">
         <is>
-          <t>shipListCode</t>
+          <t>purchaseOrderStatus</t>
         </is>
       </c>
       <c r="B239" s="4" t="inlineStr">
         <is>
-          <t>InventoryTransfers</t>
+          <t>PurchaseOrders</t>
         </is>
       </c>
       <c r="C239" s="4" t="inlineStr">
@@ -27802,7 +27810,7 @@
       </c>
       <c r="E239" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate InventoryTransfers.shipListCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate PurchaseOrders.purchaseOrderStatus?</t>
         </is>
       </c>
       <c r="F239" s="4" t="inlineStr">
@@ -27819,7 +27827,7 @@
     <row r="240">
       <c r="A240" s="4" t="inlineStr">
         <is>
-          <t>purchaseOrderNumber</t>
+          <t>creationDateTime</t>
         </is>
       </c>
       <c r="B240" s="4" t="inlineStr">
@@ -27839,7 +27847,7 @@
       </c>
       <c r="E240" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PurchaseOrders.purchaseOrderNumber?</t>
+          <t>What confirmed CoCre8/SAP source should populate PurchaseOrders.creationDateTime?</t>
         </is>
       </c>
       <c r="F240" s="4" t="inlineStr">
@@ -27856,7 +27864,7 @@
     <row r="241">
       <c r="A241" s="4" t="inlineStr">
         <is>
-          <t>purchaseOrderStatus</t>
+          <t>approvalDateTime</t>
         </is>
       </c>
       <c r="B241" s="4" t="inlineStr">
@@ -27876,7 +27884,7 @@
       </c>
       <c r="E241" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PurchaseOrders.purchaseOrderStatus?</t>
+          <t>What confirmed CoCre8/SAP source should populate PurchaseOrders.approvalDateTime?</t>
         </is>
       </c>
       <c r="F241" s="4" t="inlineStr">
@@ -27893,7 +27901,7 @@
     <row r="242">
       <c r="A242" s="4" t="inlineStr">
         <is>
-          <t>creationDateTime</t>
+          <t>toWarehouseId</t>
         </is>
       </c>
       <c r="B242" s="4" t="inlineStr">
@@ -27913,7 +27921,7 @@
       </c>
       <c r="E242" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PurchaseOrders.creationDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate PurchaseOrders.toWarehouseId?</t>
         </is>
       </c>
       <c r="F242" s="4" t="inlineStr">
@@ -27930,7 +27938,7 @@
     <row r="243">
       <c r="A243" s="4" t="inlineStr">
         <is>
-          <t>approvalDateTime</t>
+          <t>vendorId</t>
         </is>
       </c>
       <c r="B243" s="4" t="inlineStr">
@@ -27950,7 +27958,7 @@
       </c>
       <c r="E243" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PurchaseOrders.approvalDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate PurchaseOrders.vendorId?</t>
         </is>
       </c>
       <c r="F243" s="4" t="inlineStr">
@@ -27967,7 +27975,7 @@
     <row r="244">
       <c r="A244" s="4" t="inlineStr">
         <is>
-          <t>toWarehouseId</t>
+          <t>demandStatus</t>
         </is>
       </c>
       <c r="B244" s="4" t="inlineStr">
@@ -27987,7 +27995,7 @@
       </c>
       <c r="E244" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PurchaseOrders.toWarehouseId?</t>
+          <t>What confirmed CoCre8/SAP source should populate PurchaseOrders.demandStatus?</t>
         </is>
       </c>
       <c r="F244" s="4" t="inlineStr">
@@ -28004,7 +28012,7 @@
     <row r="245">
       <c r="A245" s="4" t="inlineStr">
         <is>
-          <t>vendorId</t>
+          <t>customerId</t>
         </is>
       </c>
       <c r="B245" s="4" t="inlineStr">
@@ -28024,7 +28032,7 @@
       </c>
       <c r="E245" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PurchaseOrders.vendorId?</t>
+          <t>What confirmed CoCre8/SAP source should populate PurchaseOrders.customerId?</t>
         </is>
       </c>
       <c r="F245" s="4" t="inlineStr">
@@ -28041,7 +28049,7 @@
     <row r="246">
       <c r="A246" s="4" t="inlineStr">
         <is>
-          <t>demandStatus</t>
+          <t>requestTicketDateTime</t>
         </is>
       </c>
       <c r="B246" s="4" t="inlineStr">
@@ -28061,7 +28069,7 @@
       </c>
       <c r="E246" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PurchaseOrders.demandStatus?</t>
+          <t>What confirmed CoCre8/SAP source should populate PurchaseOrders.requestTicketDateTime?</t>
         </is>
       </c>
       <c r="F246" s="4" t="inlineStr">
@@ -28078,7 +28086,7 @@
     <row r="247">
       <c r="A247" s="4" t="inlineStr">
         <is>
-          <t>customerId</t>
+          <t>isResolved</t>
         </is>
       </c>
       <c r="B247" s="4" t="inlineStr">
@@ -28098,7 +28106,7 @@
       </c>
       <c r="E247" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PurchaseOrders.customerId?</t>
+          <t>What confirmed CoCre8/SAP source should populate PurchaseOrders.isResolved?</t>
         </is>
       </c>
       <c r="F247" s="4" t="inlineStr">
@@ -28115,7 +28123,7 @@
     <row r="248">
       <c r="A248" s="4" t="inlineStr">
         <is>
-          <t>requestTicketDateTime</t>
+          <t>partNumber</t>
         </is>
       </c>
       <c r="B248" s="4" t="inlineStr">
@@ -28135,7 +28143,7 @@
       </c>
       <c r="E248" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PurchaseOrders.requestTicketDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate PurchaseOrders.partNumber?</t>
         </is>
       </c>
       <c r="F248" s="4" t="inlineStr">
@@ -28152,7 +28160,7 @@
     <row r="249">
       <c r="A249" s="4" t="inlineStr">
         <is>
-          <t>isResolved</t>
+          <t>quantity</t>
         </is>
       </c>
       <c r="B249" s="4" t="inlineStr">
@@ -28172,7 +28180,7 @@
       </c>
       <c r="E249" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PurchaseOrders.isResolved?</t>
+          <t>What confirmed CoCre8/SAP source should populate PurchaseOrders.quantity?</t>
         </is>
       </c>
       <c r="F249" s="4" t="inlineStr">
@@ -28189,7 +28197,7 @@
     <row r="250">
       <c r="A250" s="4" t="inlineStr">
         <is>
-          <t>partNumber</t>
+          <t>lineCost</t>
         </is>
       </c>
       <c r="B250" s="4" t="inlineStr">
@@ -28209,7 +28217,7 @@
       </c>
       <c r="E250" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PurchaseOrders.partNumber?</t>
+          <t>What confirmed CoCre8/SAP source should populate PurchaseOrders.lineCost?</t>
         </is>
       </c>
       <c r="F250" s="4" t="inlineStr">
@@ -28226,7 +28234,7 @@
     <row r="251">
       <c r="A251" s="4" t="inlineStr">
         <is>
-          <t>quantity</t>
+          <t>quantityReceived</t>
         </is>
       </c>
       <c r="B251" s="4" t="inlineStr">
@@ -28246,7 +28254,7 @@
       </c>
       <c r="E251" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PurchaseOrders.quantity?</t>
+          <t>What confirmed CoCre8/SAP source should populate PurchaseOrders.quantityReceived?</t>
         </is>
       </c>
       <c r="F251" s="4" t="inlineStr">
@@ -28263,7 +28271,7 @@
     <row r="252">
       <c r="A252" s="4" t="inlineStr">
         <is>
-          <t>lineCost</t>
+          <t>receivedDateTime</t>
         </is>
       </c>
       <c r="B252" s="4" t="inlineStr">
@@ -28283,7 +28291,7 @@
       </c>
       <c r="E252" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PurchaseOrders.lineCost?</t>
+          <t>What confirmed CoCre8/SAP source should populate PurchaseOrders.receivedDateTime?</t>
         </is>
       </c>
       <c r="F252" s="4" t="inlineStr">
@@ -28300,12 +28308,12 @@
     <row r="253">
       <c r="A253" s="4" t="inlineStr">
         <is>
-          <t>quantityReceived</t>
+          <t>partTypeCode</t>
         </is>
       </c>
       <c r="B253" s="4" t="inlineStr">
         <is>
-          <t>PurchaseOrders</t>
+          <t>PartTypes</t>
         </is>
       </c>
       <c r="C253" s="4" t="inlineStr">
@@ -28320,7 +28328,7 @@
       </c>
       <c r="E253" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PurchaseOrders.quantityReceived?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartTypes.partTypeCode?</t>
         </is>
       </c>
       <c r="F253" s="4" t="inlineStr">
@@ -28337,12 +28345,12 @@
     <row r="254">
       <c r="A254" s="4" t="inlineStr">
         <is>
-          <t>receivedDateTime</t>
+          <t>description</t>
         </is>
       </c>
       <c r="B254" s="4" t="inlineStr">
         <is>
-          <t>PurchaseOrders</t>
+          <t>PartTypes</t>
         </is>
       </c>
       <c r="C254" s="4" t="inlineStr">
@@ -28357,7 +28365,7 @@
       </c>
       <c r="E254" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PurchaseOrders.receivedDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartTypes.description?</t>
         </is>
       </c>
       <c r="F254" s="4" t="inlineStr">
@@ -28374,12 +28382,12 @@
     <row r="255">
       <c r="A255" s="4" t="inlineStr">
         <is>
-          <t>partTypeCode</t>
+          <t>partNumber</t>
         </is>
       </c>
       <c r="B255" s="4" t="inlineStr">
         <is>
-          <t>PartTypes</t>
+          <t>Yields</t>
         </is>
       </c>
       <c r="C255" s="4" t="inlineStr">
@@ -28394,7 +28402,7 @@
       </c>
       <c r="E255" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartTypes.partTypeCode?</t>
+          <t>What confirmed CoCre8/SAP source should populate Yields.partNumber?</t>
         </is>
       </c>
       <c r="F255" s="4" t="inlineStr">
@@ -28411,12 +28419,12 @@
     <row r="256">
       <c r="A256" s="4" t="inlineStr">
         <is>
-          <t>description</t>
+          <t>unitOfMeasure</t>
         </is>
       </c>
       <c r="B256" s="4" t="inlineStr">
         <is>
-          <t>PartTypes</t>
+          <t>Yields</t>
         </is>
       </c>
       <c r="C256" s="4" t="inlineStr">
@@ -28431,7 +28439,7 @@
       </c>
       <c r="E256" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PartTypes.description?</t>
+          <t>What confirmed CoCre8/SAP source should populate Yields.unitOfMeasure?</t>
         </is>
       </c>
       <c r="F256" s="4" t="inlineStr">
@@ -28448,7 +28456,7 @@
     <row r="257">
       <c r="A257" s="4" t="inlineStr">
         <is>
-          <t>partNumber</t>
+          <t>yield</t>
         </is>
       </c>
       <c r="B257" s="4" t="inlineStr">
@@ -28468,7 +28476,7 @@
       </c>
       <c r="E257" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Yields.partNumber?</t>
+          <t>What confirmed CoCre8/SAP source should populate Yields.yield?</t>
         </is>
       </c>
       <c r="F257" s="4" t="inlineStr">
@@ -28485,12 +28493,12 @@
     <row r="258">
       <c r="A258" s="4" t="inlineStr">
         <is>
-          <t>unitOfMeasure</t>
+          <t>actionGroupId</t>
         </is>
       </c>
       <c r="B258" s="4" t="inlineStr">
         <is>
-          <t>Yields</t>
+          <t>ActionGroups</t>
         </is>
       </c>
       <c r="C258" s="4" t="inlineStr">
@@ -28505,7 +28513,7 @@
       </c>
       <c r="E258" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Yields.unitOfMeasure?</t>
+          <t>What confirmed CoCre8/SAP source should populate ActionGroups.actionGroupId?</t>
         </is>
       </c>
       <c r="F258" s="4" t="inlineStr">
@@ -28522,12 +28530,12 @@
     <row r="259">
       <c r="A259" s="4" t="inlineStr">
         <is>
-          <t>yield</t>
+          <t>nodeId</t>
         </is>
       </c>
       <c r="B259" s="4" t="inlineStr">
         <is>
-          <t>Yields</t>
+          <t>ActionGroups</t>
         </is>
       </c>
       <c r="C259" s="4" t="inlineStr">
@@ -28542,7 +28550,7 @@
       </c>
       <c r="E259" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate Yields.yield?</t>
+          <t>What confirmed CoCre8/SAP source should populate ActionGroups.nodeId?</t>
         </is>
       </c>
       <c r="F259" s="4" t="inlineStr">
@@ -28559,7 +28567,7 @@
     <row r="260">
       <c r="A260" s="4" t="inlineStr">
         <is>
-          <t>actionGroupId</t>
+          <t>actionGroupDescription</t>
         </is>
       </c>
       <c r="B260" s="4" t="inlineStr">
@@ -28579,7 +28587,7 @@
       </c>
       <c r="E260" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ActionGroups.actionGroupId?</t>
+          <t>What confirmed CoCre8/SAP source should populate ActionGroups.actionGroupDescription?</t>
         </is>
       </c>
       <c r="F260" s="4" t="inlineStr">
@@ -28596,7 +28604,7 @@
     <row r="261">
       <c r="A261" s="4" t="inlineStr">
         <is>
-          <t>nodeId</t>
+          <t>assignAnySkill</t>
         </is>
       </c>
       <c r="B261" s="4" t="inlineStr">
@@ -28616,7 +28624,7 @@
       </c>
       <c r="E261" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ActionGroups.nodeId?</t>
+          <t>What confirmed CoCre8/SAP source should populate ActionGroups.assignAnySkill?</t>
         </is>
       </c>
       <c r="F261" s="4" t="inlineStr">
@@ -28633,7 +28641,7 @@
     <row r="262">
       <c r="A262" s="4" t="inlineStr">
         <is>
-          <t>actionGroupDescription</t>
+          <t>isUsed</t>
         </is>
       </c>
       <c r="B262" s="4" t="inlineStr">
@@ -28653,7 +28661,7 @@
       </c>
       <c r="E262" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ActionGroups.actionGroupDescription?</t>
+          <t>What confirmed CoCre8/SAP source should populate ActionGroups.isUsed?</t>
         </is>
       </c>
       <c r="F262" s="4" t="inlineStr">
@@ -28670,7 +28678,7 @@
     <row r="263">
       <c r="A263" s="4" t="inlineStr">
         <is>
-          <t>assignAnySkill</t>
+          <t>isObsolete</t>
         </is>
       </c>
       <c r="B263" s="4" t="inlineStr">
@@ -28690,7 +28698,7 @@
       </c>
       <c r="E263" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ActionGroups.assignAnySkill?</t>
+          <t>What confirmed CoCre8/SAP source should populate ActionGroups.isObsolete?</t>
         </is>
       </c>
       <c r="F263" s="4" t="inlineStr">
@@ -28707,12 +28715,12 @@
     <row r="264">
       <c r="A264" s="4" t="inlineStr">
         <is>
-          <t>isUsed</t>
+          <t>warehouseId</t>
         </is>
       </c>
       <c r="B264" s="4" t="inlineStr">
         <is>
-          <t>ActionGroups</t>
+          <t>WarehouseExclusions</t>
         </is>
       </c>
       <c r="C264" s="4" t="inlineStr">
@@ -28727,7 +28735,7 @@
       </c>
       <c r="E264" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ActionGroups.isUsed?</t>
+          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.warehouseId?</t>
         </is>
       </c>
       <c r="F264" s="4" t="inlineStr">
@@ -28744,12 +28752,12 @@
     <row r="265">
       <c r="A265" s="4" t="inlineStr">
         <is>
-          <t>isObsolete</t>
+          <t>exclusionType</t>
         </is>
       </c>
       <c r="B265" s="4" t="inlineStr">
         <is>
-          <t>ActionGroups</t>
+          <t>WarehouseExclusions</t>
         </is>
       </c>
       <c r="C265" s="4" t="inlineStr">
@@ -28764,7 +28772,7 @@
       </c>
       <c r="E265" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate ActionGroups.isObsolete?</t>
+          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.exclusionType?</t>
         </is>
       </c>
       <c r="F265" s="4" t="inlineStr">
@@ -28781,7 +28789,7 @@
     <row r="266">
       <c r="A266" s="4" t="inlineStr">
         <is>
-          <t>warehouseId</t>
+          <t>exclusion</t>
         </is>
       </c>
       <c r="B266" s="4" t="inlineStr">
@@ -28801,7 +28809,7 @@
       </c>
       <c r="E266" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.warehouseId?</t>
+          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.exclusion?</t>
         </is>
       </c>
       <c r="F266" s="4" t="inlineStr">
@@ -28815,82 +28823,8 @@
         </is>
       </c>
     </row>
-    <row r="267">
-      <c r="A267" s="4" t="inlineStr">
-        <is>
-          <t>exclusionType</t>
-        </is>
-      </c>
-      <c r="B267" s="4" t="inlineStr">
-        <is>
-          <t>WarehouseExclusions</t>
-        </is>
-      </c>
-      <c r="C267" s="4" t="inlineStr">
-        <is>
-          <t>Planning V2 template</t>
-        </is>
-      </c>
-      <c r="D267" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="E267" s="4" t="inlineStr">
-        <is>
-          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.exclusionType?</t>
-        </is>
-      </c>
-      <c r="F267" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP Service Layer first; only use external/manual source if SAP cannot supply it.</t>
-        </is>
-      </c>
-      <c r="G267" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="268">
-      <c r="A268" s="4" t="inlineStr">
-        <is>
-          <t>exclusion</t>
-        </is>
-      </c>
-      <c r="B268" s="4" t="inlineStr">
-        <is>
-          <t>WarehouseExclusions</t>
-        </is>
-      </c>
-      <c r="C268" s="4" t="inlineStr">
-        <is>
-          <t>Planning V2 template</t>
-        </is>
-      </c>
-      <c r="D268" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="E268" s="4" t="inlineStr">
-        <is>
-          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.exclusion?</t>
-        </is>
-      </c>
-      <c r="F268" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP Service Layer first; only use external/manual source if SAP cannot supply it.</t>
-        </is>
-      </c>
-      <c r="G268" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:G268"/>
+  <autoFilter ref="A1:G266"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -29391,7 +29325,7 @@
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>isPrimary; primaryPartNumber; isBranchStockable; isBootStockable; productClass; productType; costCategory; partType; isKit; isObsolete; isService; isTool; isExcludeFromReplenishment; isSmallPart; purchaseLeadTimeDays; isCritical</t>
+          <t>isBranchStockable; isBootStockable; productClass; productType; costCategory; partType; isKit; isObsolete; isService; isTool; isExcludeFromReplenishment; isSmallPart; purchaseLeadTimeDays; isCritical</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record SAP item group investigation for part classifications
</commit_message>
<xml_diff>
--- a/docs/field-map/CoCre8_PlanningV2_Template_Field_Map.xlsx
+++ b/docs/field-map/CoCre8_PlanningV2_Template_Field_Map.xlsx
@@ -17,7 +17,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Target Fields'!$A$1:$P$153</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Template Fields'!$A$1:$H$180</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Source Evidence'!$A$1:$D$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Source Evidence'!$A$1:$D$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Unknowns'!$A$1:$G$266</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Output Objects'!$A$1:$E$34</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'SAP Investigation Log'!$A$1:$E$10</definedName>
@@ -218,8 +218,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourceEvidence" displayName="SourceEvidence" ref="A1:D12" headerRowCount="1">
-  <autoFilter ref="A1:D12"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourceEvidence" displayName="SourceEvidence" ref="A1:D13" headerRowCount="1">
+  <autoFilter ref="A1:D13"/>
   <tableColumns count="4">
     <tableColumn id="1" name="Source"/>
     <tableColumn id="2" name="Path"/>
@@ -12408,7 +12408,7 @@
     <col width="28" customWidth="1" min="2" max="2"/>
     <col width="23" customWidth="1" min="3" max="3"/>
     <col width="62" customWidth="1" min="4" max="4"/>
-    <col width="23" customWidth="1" min="5" max="5"/>
+    <col width="33" customWidth="1" min="5" max="5"/>
     <col width="62" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="62" customWidth="1" min="8" max="8"/>
@@ -13263,7 +13263,7 @@
       <c r="D24" s="4" t="inlineStr"/>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>Investigate SAP first</t>
+          <t>Not available in checked source</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr"/>
@@ -13274,7 +13274,7 @@
       </c>
       <c r="H24" s="4" t="inlineStr">
         <is>
-          <t>Left blank. CoCre8 local reporting has only item group codes; live SAP ItemGroups/OITM needs investigation for class/type semantics.</t>
+          <t>Left blank. Live SAP item master check found broad ItemGroups such as FUJITSU/ACER/CHOICE and generic ItemType/ItemClass/MaterialType values, not Planning V2 class/type semantics.</t>
         </is>
       </c>
     </row>
@@ -13297,7 +13297,7 @@
       <c r="D25" s="4" t="inlineStr"/>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>Investigate SAP first</t>
+          <t>Not available in checked source</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr"/>
@@ -13308,7 +13308,7 @@
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>Left blank. CoCre8 local reporting has only item group codes; live SAP ItemGroups/OITM needs investigation for class/type semantics.</t>
+          <t>Left blank. Live SAP item master check found broad ItemGroups such as FUJITSU/ACER/CHOICE and generic ItemType/ItemClass/MaterialType values, not Planning V2 class/type semantics.</t>
         </is>
       </c>
     </row>
@@ -13365,7 +13365,7 @@
       <c r="D27" s="4" t="inlineStr"/>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>Investigate SAP first</t>
+          <t>Not available in checked source</t>
         </is>
       </c>
       <c r="F27" s="4" t="inlineStr"/>
@@ -13376,7 +13376,7 @@
       </c>
       <c r="H27" s="4" t="inlineStr">
         <is>
-          <t>Left blank. CoCre8 local reporting has only item group codes; live SAP ItemGroups/OITM needs investigation for class/type semantics.</t>
+          <t>Left blank. Live SAP item master check found broad ItemGroups such as FUJITSU/ACER/CHOICE and generic ItemType/ItemClass/MaterialType values, not Planning V2 class/type semantics.</t>
         </is>
       </c>
     </row>
@@ -18681,7 +18681,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -18954,8 +18954,30 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Live SAP item group check</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>MinStock3 SAP Service Layer credentials</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Checked Items and ItemGroups while VPN was connected. ItemGroups are broad customer/manufacturer groups such as FUJITSU, ACER, and CHOICE; sampled item master fields ItemType, ItemClass, and MaterialType are generic SAP classifications.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D12"/>
+  <autoFilter ref="A1:D13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -18975,7 +18997,7 @@
     <col width="29" customWidth="1" min="1" max="1"/>
     <col width="62" customWidth="1" min="2" max="2"/>
     <col width="53" customWidth="1" min="3" max="3"/>
-    <col width="23" customWidth="1" min="4" max="4"/>
+    <col width="33" customWidth="1" min="4" max="4"/>
     <col width="62" customWidth="1" min="5" max="5"/>
     <col width="62" customWidth="1" min="6" max="6"/>
     <col width="62" customWidth="1" min="7" max="7"/>
@@ -23328,7 +23350,7 @@
       </c>
       <c r="D118" s="4" t="inlineStr">
         <is>
-          <t>Investigate SAP first</t>
+          <t>Not available in checked source</t>
         </is>
       </c>
       <c r="E118" s="4" t="inlineStr">
@@ -23343,7 +23365,7 @@
       </c>
       <c r="G118" s="4" t="inlineStr">
         <is>
-          <t>Left blank. CoCre8 local reporting has only item group codes; live SAP ItemGroups/OITM needs investigation for class/type semantics.</t>
+          <t>Left blank. Live SAP item master check found broad ItemGroups such as FUJITSU/ACER/CHOICE and generic ItemType/ItemClass/MaterialType values, not Planning V2 class/type semantics.</t>
         </is>
       </c>
     </row>
@@ -23365,7 +23387,7 @@
       </c>
       <c r="D119" s="4" t="inlineStr">
         <is>
-          <t>Investigate SAP first</t>
+          <t>Not available in checked source</t>
         </is>
       </c>
       <c r="E119" s="4" t="inlineStr">
@@ -23380,7 +23402,7 @@
       </c>
       <c r="G119" s="4" t="inlineStr">
         <is>
-          <t>Left blank. CoCre8 local reporting has only item group codes; live SAP ItemGroups/OITM needs investigation for class/type semantics.</t>
+          <t>Left blank. Live SAP item master check found broad ItemGroups such as FUJITSU/ACER/CHOICE and generic ItemType/ItemClass/MaterialType values, not Planning V2 class/type semantics.</t>
         </is>
       </c>
     </row>
@@ -23439,7 +23461,7 @@
       </c>
       <c r="D121" s="4" t="inlineStr">
         <is>
-          <t>Investigate SAP first</t>
+          <t>Not available in checked source</t>
         </is>
       </c>
       <c r="E121" s="4" t="inlineStr">
@@ -23454,7 +23476,7 @@
       </c>
       <c r="G121" s="4" t="inlineStr">
         <is>
-          <t>Left blank. CoCre8 local reporting has only item group codes; live SAP ItemGroups/OITM needs investigation for class/type semantics.</t>
+          <t>Left blank. Live SAP item master check found broad ItemGroups such as FUJITSU/ACER/CHOICE and generic ItemType/ItemClass/MaterialType values, not Planning V2 class/type semantics.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Clarify customer and warehouse template gaps
</commit_message>
<xml_diff>
--- a/docs/field-map/CoCre8_PlanningV2_Template_Field_Map.xlsx
+++ b/docs/field-map/CoCre8_PlanningV2_Template_Field_Map.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Target Fields" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Template Fields" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Source Evidence" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Unknowns" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Output Objects" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="SAP Investigation Log" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Target Fields" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Template Fields" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Evidence" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unknowns" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Output Objects" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SAP Investigation Log" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Target Fields'!$A$1:$P$153</definedName>
@@ -12623,7 +12623,7 @@
       <c r="D6" s="4" t="inlineStr"/>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Investigate SAP first</t>
+          <t>Investigate source</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr"/>
@@ -12634,7 +12634,7 @@
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+          <t>Left blank. User has no confirmed source yet for customer grouping.</t>
         </is>
       </c>
     </row>
@@ -12695,7 +12695,7 @@
       <c r="D8" s="4" t="inlineStr"/>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Investigate SAP first</t>
+          <t>Investigate source</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr"/>
@@ -12706,7 +12706,7 @@
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+          <t>Left blank. User has no confirmed source yet for customer skill assignment rules.</t>
         </is>
       </c>
     </row>
@@ -12729,7 +12729,7 @@
       <c r="D9" s="4" t="inlineStr"/>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Investigate SAP first</t>
+          <t>Investigate source</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr"/>
@@ -12740,7 +12740,7 @@
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+          <t>Left blank. User has no confirmed source yet for customer active/inactive status.</t>
         </is>
       </c>
     </row>
@@ -12763,7 +12763,7 @@
       <c r="D10" s="4" t="inlineStr"/>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>Investigate SAP first</t>
+          <t>Investigate source</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr"/>
@@ -12774,7 +12774,7 @@
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+          <t>Left blank. User has no confirmed source yet for SLA cost.</t>
         </is>
       </c>
     </row>
@@ -12797,7 +12797,7 @@
       <c r="D11" s="4" t="inlineStr"/>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>Investigate SAP first</t>
+          <t>Investigate source</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr"/>
@@ -12808,7 +12808,7 @@
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+          <t>Left blank. User has no confirmed source yet for SLA revenue.</t>
         </is>
       </c>
     </row>
@@ -12831,7 +12831,7 @@
       <c r="D12" s="4" t="inlineStr"/>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Investigate SAP first</t>
+          <t>Investigate source</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr"/>
@@ -12842,7 +12842,7 @@
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+          <t>Left blank. User has no confirmed source yet for standard response time.</t>
         </is>
       </c>
     </row>
@@ -12865,7 +12865,7 @@
       <c r="D13" s="4" t="inlineStr"/>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>Investigate SAP first</t>
+          <t>Investigate source</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr"/>
@@ -12876,7 +12876,7 @@
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+          <t>Left blank. User has no confirmed source yet for standard repair time.</t>
         </is>
       </c>
     </row>
@@ -14144,7 +14144,7 @@
       </c>
       <c r="H49" s="4" t="inlineStr">
         <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+          <t>Expected site/address id linking to the Addresses template. Data dictionary field: warehouse.address_id.</t>
         </is>
       </c>
     </row>
@@ -14182,7 +14182,7 @@
       </c>
       <c r="H50" s="4" t="inlineStr">
         <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+          <t>Expected associated planning hierarchy node id. Data fields list this as warehouse.node_id / associated node.</t>
         </is>
       </c>
     </row>
@@ -14220,7 +14220,7 @@
       </c>
       <c r="H51" s="4" t="inlineStr">
         <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+          <t>Expected preferred warehouse for return/faulty stock going to repair or scrap. Data fields: return_warehouse.</t>
         </is>
       </c>
     </row>
@@ -14258,7 +14258,7 @@
       </c>
       <c r="H52" s="4" t="inlineStr">
         <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+          <t>Expected preferred replenishment/source warehouse. Data fields: supply_warehouse.</t>
         </is>
       </c>
     </row>
@@ -14296,7 +14296,7 @@
       </c>
       <c r="H53" s="4" t="inlineStr">
         <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+          <t>Expected site type enum; sample template uses BOOT, DEP, and REPAIR. Data fields mark warehouse_type_id as critical.</t>
         </is>
       </c>
     </row>
@@ -14368,7 +14368,7 @@
       </c>
       <c r="H55" s="4" t="inlineStr">
         <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+          <t>Expected true when this is an internal repair location. Data dictionary field: is_repair_whse.</t>
         </is>
       </c>
     </row>
@@ -14402,7 +14402,7 @@
       </c>
       <c r="H56" s="4" t="inlineStr">
         <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+          <t>Expected true when the site can be restocked. Data dictionary field: is_replenishable.</t>
         </is>
       </c>
     </row>
@@ -14436,7 +14436,7 @@
       </c>
       <c r="H57" s="4" t="inlineStr">
         <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+          <t>Expected true when technician/boot location can accept stock. Data fields: cst_boot_stockable.</t>
         </is>
       </c>
     </row>
@@ -14470,7 +14470,7 @@
       </c>
       <c r="H58" s="4" t="inlineStr">
         <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+          <t>Expected true when branch/regional location can accept stock. Data fields: cst_branch_stockable.</t>
         </is>
       </c>
     </row>
@@ -14504,7 +14504,7 @@
       </c>
       <c r="H59" s="4" t="inlineStr">
         <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+          <t>Expected true when this is an outlying/regional location. Data fields: cst_remote.</t>
         </is>
       </c>
     </row>
@@ -14542,7 +14542,7 @@
       </c>
       <c r="H60" s="4" t="inlineStr">
         <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+          <t>Expected current/inactive status if required by the importer. Template says confirm; data fields mention cst_active and is_obsolete.</t>
         </is>
       </c>
     </row>
@@ -22906,7 +22906,7 @@
       </c>
       <c r="D106" s="4" t="inlineStr">
         <is>
-          <t>Investigate SAP first</t>
+          <t>Investigate source</t>
         </is>
       </c>
       <c r="E106" s="4" t="inlineStr">
@@ -22921,7 +22921,7 @@
       </c>
       <c r="G106" s="4" t="inlineStr">
         <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+          <t>Left blank. User has no confirmed source yet for customer grouping.</t>
         </is>
       </c>
     </row>
@@ -22943,7 +22943,7 @@
       </c>
       <c r="D107" s="4" t="inlineStr">
         <is>
-          <t>Investigate SAP first</t>
+          <t>Investigate source</t>
         </is>
       </c>
       <c r="E107" s="4" t="inlineStr">
@@ -22958,7 +22958,7 @@
       </c>
       <c r="G107" s="4" t="inlineStr">
         <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+          <t>Left blank. User has no confirmed source yet for customer skill assignment rules.</t>
         </is>
       </c>
     </row>
@@ -22980,7 +22980,7 @@
       </c>
       <c r="D108" s="4" t="inlineStr">
         <is>
-          <t>Investigate SAP first</t>
+          <t>Investigate source</t>
         </is>
       </c>
       <c r="E108" s="4" t="inlineStr">
@@ -22995,7 +22995,7 @@
       </c>
       <c r="G108" s="4" t="inlineStr">
         <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+          <t>Left blank. User has no confirmed source yet for customer active/inactive status.</t>
         </is>
       </c>
     </row>
@@ -23017,7 +23017,7 @@
       </c>
       <c r="D109" s="4" t="inlineStr">
         <is>
-          <t>Investigate SAP first</t>
+          <t>Investigate source</t>
         </is>
       </c>
       <c r="E109" s="4" t="inlineStr">
@@ -23032,7 +23032,7 @@
       </c>
       <c r="G109" s="4" t="inlineStr">
         <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+          <t>Left blank. User has no confirmed source yet for SLA cost.</t>
         </is>
       </c>
     </row>
@@ -23054,7 +23054,7 @@
       </c>
       <c r="D110" s="4" t="inlineStr">
         <is>
-          <t>Investigate SAP first</t>
+          <t>Investigate source</t>
         </is>
       </c>
       <c r="E110" s="4" t="inlineStr">
@@ -23069,7 +23069,7 @@
       </c>
       <c r="G110" s="4" t="inlineStr">
         <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+          <t>Left blank. User has no confirmed source yet for SLA revenue.</t>
         </is>
       </c>
     </row>
@@ -23091,7 +23091,7 @@
       </c>
       <c r="D111" s="4" t="inlineStr">
         <is>
-          <t>Investigate SAP first</t>
+          <t>Investigate source</t>
         </is>
       </c>
       <c r="E111" s="4" t="inlineStr">
@@ -23106,7 +23106,7 @@
       </c>
       <c r="G111" s="4" t="inlineStr">
         <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+          <t>Left blank. User has no confirmed source yet for standard response time.</t>
         </is>
       </c>
     </row>
@@ -23128,7 +23128,7 @@
       </c>
       <c r="D112" s="4" t="inlineStr">
         <is>
-          <t>Investigate SAP first</t>
+          <t>Investigate source</t>
         </is>
       </c>
       <c r="E112" s="4" t="inlineStr">
@@ -23143,7 +23143,7 @@
       </c>
       <c r="G112" s="4" t="inlineStr">
         <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+          <t>Left blank. User has no confirmed source yet for standard repair time.</t>
         </is>
       </c>
     </row>
@@ -24253,7 +24253,7 @@
       </c>
       <c r="G142" s="4" t="inlineStr">
         <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+          <t>Expected site/address id linking to the Addresses template. Data dictionary field: warehouse.address_id.</t>
         </is>
       </c>
     </row>
@@ -24290,7 +24290,7 @@
       </c>
       <c r="G143" s="4" t="inlineStr">
         <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+          <t>Expected associated planning hierarchy node id. Data fields list this as warehouse.node_id / associated node.</t>
         </is>
       </c>
     </row>
@@ -24327,7 +24327,7 @@
       </c>
       <c r="G144" s="4" t="inlineStr">
         <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+          <t>Expected preferred warehouse for return/faulty stock going to repair or scrap. Data fields: return_warehouse.</t>
         </is>
       </c>
     </row>
@@ -24364,7 +24364,7 @@
       </c>
       <c r="G145" s="4" t="inlineStr">
         <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+          <t>Expected preferred replenishment/source warehouse. Data fields: supply_warehouse.</t>
         </is>
       </c>
     </row>
@@ -24401,7 +24401,7 @@
       </c>
       <c r="G146" s="4" t="inlineStr">
         <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+          <t>Expected site type enum; sample template uses BOOT, DEP, and REPAIR. Data fields mark warehouse_type_id as critical.</t>
         </is>
       </c>
     </row>
@@ -24438,7 +24438,7 @@
       </c>
       <c r="G147" s="4" t="inlineStr">
         <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+          <t>Expected true when this is an internal repair location. Data dictionary field: is_repair_whse.</t>
         </is>
       </c>
     </row>
@@ -24475,7 +24475,7 @@
       </c>
       <c r="G148" s="4" t="inlineStr">
         <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+          <t>Expected true when the site can be restocked. Data dictionary field: is_replenishable.</t>
         </is>
       </c>
     </row>
@@ -24512,7 +24512,7 @@
       </c>
       <c r="G149" s="4" t="inlineStr">
         <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+          <t>Expected true when technician/boot location can accept stock. Data fields: cst_boot_stockable.</t>
         </is>
       </c>
     </row>
@@ -24549,7 +24549,7 @@
       </c>
       <c r="G150" s="4" t="inlineStr">
         <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+          <t>Expected true when branch/regional location can accept stock. Data fields: cst_branch_stockable.</t>
         </is>
       </c>
     </row>
@@ -24586,7 +24586,7 @@
       </c>
       <c r="G151" s="4" t="inlineStr">
         <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+          <t>Expected true when this is an outlying/regional location. Data fields: cst_remote.</t>
         </is>
       </c>
     </row>
@@ -24623,7 +24623,7 @@
       </c>
       <c r="G152" s="4" t="inlineStr">
         <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+          <t>Expected current/inactive status if required by the importer. Template says confirm; data fields mention cst_active and is_obsolete.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Populate purchase order template from SAP
</commit_message>
<xml_diff>
--- a/docs/field-map/CoCre8_PlanningV2_Template_Field_Map.xlsx
+++ b/docs/field-map/CoCre8_PlanningV2_Template_Field_Map.xlsx
@@ -18,7 +18,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Target Fields'!$A$1:$P$151</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Template Fields'!$A$1:$H$180</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Source Evidence'!$A$1:$D$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Unknowns'!$A$1:$G$249</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Unknowns'!$A$1:$G$235</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Output Objects'!$A$1:$E$34</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'SAP Investigation Log'!$A$1:$E$10</definedName>
   </definedNames>
@@ -239,8 +239,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Unknowns" displayName="Unknowns" ref="A1:G249" headerRowCount="1">
-  <autoFilter ref="A1:G249"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Unknowns" displayName="Unknowns" ref="A1:G235" headerRowCount="1">
+  <autoFilter ref="A1:G235"/>
   <tableColumns count="7">
     <tableColumn id="1" name="Field"/>
     <tableColumn id="2" name="Object"/>
@@ -17917,206 +17917,230 @@
       </c>
     </row>
     <row r="152">
-      <c r="A152" s="4" t="inlineStr">
+      <c r="A152" s="2" t="inlineStr">
         <is>
           <t>PurchaseOrders</t>
         </is>
       </c>
-      <c r="B152" s="4" t="inlineStr">
+      <c r="B152" s="2" t="inlineStr">
         <is>
           <t>purchaseOrderNumber</t>
         </is>
       </c>
-      <c r="C152" s="4" t="inlineStr">
+      <c r="C152" s="2" t="inlineStr">
         <is>
           <t>String</t>
         </is>
       </c>
-      <c r="D152" s="4" t="inlineStr"/>
-      <c r="E152" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F152" s="4" t="inlineStr"/>
-      <c r="G152" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H152" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+      <c r="D152" s="2" t="inlineStr"/>
+      <c r="E152" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="F152" s="2" t="inlineStr">
+        <is>
+          <t>SAP Service Layer SQLQueries:OPOR.DocNum</t>
+        </is>
+      </c>
+      <c r="G152" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H152" s="2" t="inlineStr">
+        <is>
+          <t>Populated in template CSV from confirmed live SAP Service Layer or allowed SPI source.</t>
         </is>
       </c>
     </row>
     <row r="153">
-      <c r="A153" s="4" t="inlineStr">
+      <c r="A153" s="2" t="inlineStr">
         <is>
           <t>PurchaseOrders</t>
         </is>
       </c>
-      <c r="B153" s="4" t="inlineStr">
+      <c r="B153" s="2" t="inlineStr">
         <is>
           <t>purchaseOrderStatus</t>
         </is>
       </c>
-      <c r="C153" s="4" t="inlineStr">
+      <c r="C153" s="2" t="inlineStr">
         <is>
           <t>Enum&lt;String&gt;</t>
         </is>
       </c>
-      <c r="D153" s="4" t="inlineStr"/>
-      <c r="E153" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F153" s="4" t="inlineStr"/>
-      <c r="G153" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H153" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+      <c r="D153" s="2" t="inlineStr"/>
+      <c r="E153" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="F153" s="2" t="inlineStr">
+        <is>
+          <t>SAP Service Layer SQLQueries:OPOR.DocStatus/CANCELED mapped to template status</t>
+        </is>
+      </c>
+      <c r="G153" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H153" s="2" t="inlineStr">
+        <is>
+          <t>Populated in template CSV from confirmed live SAP Service Layer or allowed SPI source.</t>
         </is>
       </c>
     </row>
     <row r="154">
-      <c r="A154" s="4" t="inlineStr">
+      <c r="A154" s="2" t="inlineStr">
         <is>
           <t>PurchaseOrders</t>
         </is>
       </c>
-      <c r="B154" s="4" t="inlineStr">
+      <c r="B154" s="2" t="inlineStr">
         <is>
           <t>creationDateTime</t>
         </is>
       </c>
-      <c r="C154" s="4" t="inlineStr">
+      <c r="C154" s="2" t="inlineStr">
         <is>
           <t>Datetime</t>
         </is>
       </c>
-      <c r="D154" s="4" t="inlineStr"/>
-      <c r="E154" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F154" s="4" t="inlineStr"/>
-      <c r="G154" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H154" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+      <c r="D154" s="2" t="inlineStr"/>
+      <c r="E154" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="F154" s="2" t="inlineStr">
+        <is>
+          <t>SAP Service Layer SQLQueries:OPOR.CreateDate</t>
+        </is>
+      </c>
+      <c r="G154" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H154" s="2" t="inlineStr">
+        <is>
+          <t>Populated in template CSV from confirmed live SAP Service Layer or allowed SPI source.</t>
         </is>
       </c>
     </row>
     <row r="155">
-      <c r="A155" s="4" t="inlineStr">
+      <c r="A155" s="2" t="inlineStr">
         <is>
           <t>PurchaseOrders</t>
         </is>
       </c>
-      <c r="B155" s="4" t="inlineStr">
+      <c r="B155" s="2" t="inlineStr">
         <is>
           <t>approvalDateTime</t>
         </is>
       </c>
-      <c r="C155" s="4" t="inlineStr">
+      <c r="C155" s="2" t="inlineStr">
         <is>
           <t>Datetime</t>
         </is>
       </c>
-      <c r="D155" s="4" t="inlineStr"/>
-      <c r="E155" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F155" s="4" t="inlineStr"/>
-      <c r="G155" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H155" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+      <c r="D155" s="2" t="inlineStr"/>
+      <c r="E155" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="F155" s="2" t="inlineStr">
+        <is>
+          <t>SAP Service Layer SQLQueries:OPOR.DocDate</t>
+        </is>
+      </c>
+      <c r="G155" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H155" s="2" t="inlineStr">
+        <is>
+          <t>Populated in template CSV from confirmed live SAP Service Layer or allowed SPI source.</t>
         </is>
       </c>
     </row>
     <row r="156">
-      <c r="A156" s="4" t="inlineStr">
+      <c r="A156" s="2" t="inlineStr">
         <is>
           <t>PurchaseOrders</t>
         </is>
       </c>
-      <c r="B156" s="4" t="inlineStr">
+      <c r="B156" s="2" t="inlineStr">
         <is>
           <t>toWarehouseId</t>
         </is>
       </c>
-      <c r="C156" s="4" t="inlineStr">
+      <c r="C156" s="2" t="inlineStr">
         <is>
           <t>String</t>
         </is>
       </c>
-      <c r="D156" s="4" t="inlineStr"/>
-      <c r="E156" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F156" s="4" t="inlineStr"/>
-      <c r="G156" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H156" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+      <c r="D156" s="2" t="inlineStr"/>
+      <c r="E156" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="F156" s="2" t="inlineStr">
+        <is>
+          <t>SAP Service Layer SQLQueries:POR1.WhsCode</t>
+        </is>
+      </c>
+      <c r="G156" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H156" s="2" t="inlineStr">
+        <is>
+          <t>Populated in template CSV from confirmed live SAP Service Layer or allowed SPI source.</t>
         </is>
       </c>
     </row>
     <row r="157">
-      <c r="A157" s="4" t="inlineStr">
+      <c r="A157" s="2" t="inlineStr">
         <is>
           <t>PurchaseOrders</t>
         </is>
       </c>
-      <c r="B157" s="4" t="inlineStr">
+      <c r="B157" s="2" t="inlineStr">
         <is>
           <t>vendorId</t>
         </is>
       </c>
-      <c r="C157" s="4" t="inlineStr">
+      <c r="C157" s="2" t="inlineStr">
         <is>
           <t>String</t>
         </is>
       </c>
-      <c r="D157" s="4" t="inlineStr"/>
-      <c r="E157" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F157" s="4" t="inlineStr"/>
-      <c r="G157" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H157" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+      <c r="D157" s="2" t="inlineStr"/>
+      <c r="E157" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="F157" s="2" t="inlineStr">
+        <is>
+          <t>SAP Service Layer SQLQueries:OPOR.CardCode</t>
+        </is>
+      </c>
+      <c r="G157" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H157" s="2" t="inlineStr">
+        <is>
+          <t>Populated in template CSV from confirmed live SAP Service Layer or allowed SPI source.</t>
         </is>
       </c>
     </row>
@@ -18155,274 +18179,282 @@
       </c>
     </row>
     <row r="159">
-      <c r="A159" s="4" t="inlineStr">
+      <c r="A159" s="5" t="inlineStr">
         <is>
           <t>PurchaseOrders</t>
         </is>
       </c>
-      <c r="B159" s="4" t="inlineStr">
+      <c r="B159" s="5" t="inlineStr">
         <is>
           <t>customerId</t>
         </is>
       </c>
-      <c r="C159" s="4" t="inlineStr">
+      <c r="C159" s="5" t="inlineStr">
         <is>
           <t>String</t>
         </is>
       </c>
-      <c r="D159" s="4" t="inlineStr"/>
-      <c r="E159" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F159" s="4" t="inlineStr"/>
-      <c r="G159" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H159" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+      <c r="D159" s="5" t="inlineStr"/>
+      <c r="E159" s="5" t="inlineStr">
+        <is>
+          <t>Out of v1 scope</t>
+        </is>
+      </c>
+      <c r="F159" s="5" t="inlineStr"/>
+      <c r="G159" s="5" t="inlineStr"/>
+      <c r="H159" s="5" t="inlineStr">
+        <is>
+          <t>No corresponding purchase_orders field is marked needed for CoCre8 in the edited reference workbook.</t>
         </is>
       </c>
     </row>
     <row r="160">
-      <c r="A160" s="4" t="inlineStr">
+      <c r="A160" s="5" t="inlineStr">
         <is>
           <t>PurchaseOrders</t>
         </is>
       </c>
-      <c r="B160" s="4" t="inlineStr">
+      <c r="B160" s="5" t="inlineStr">
         <is>
           <t>requestTicketDateTime</t>
         </is>
       </c>
-      <c r="C160" s="4" t="inlineStr">
+      <c r="C160" s="5" t="inlineStr">
         <is>
           <t>Datetime</t>
         </is>
       </c>
-      <c r="D160" s="4" t="inlineStr"/>
-      <c r="E160" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F160" s="4" t="inlineStr"/>
-      <c r="G160" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H160" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+      <c r="D160" s="5" t="inlineStr"/>
+      <c r="E160" s="5" t="inlineStr">
+        <is>
+          <t>Out of v1 scope</t>
+        </is>
+      </c>
+      <c r="F160" s="5" t="inlineStr"/>
+      <c r="G160" s="5" t="inlineStr"/>
+      <c r="H160" s="5" t="inlineStr">
+        <is>
+          <t>No corresponding purchase_orders field is marked needed for CoCre8 in the edited reference workbook.</t>
         </is>
       </c>
     </row>
     <row r="161">
-      <c r="A161" s="4" t="inlineStr">
+      <c r="A161" s="5" t="inlineStr">
         <is>
           <t>PurchaseOrders</t>
         </is>
       </c>
-      <c r="B161" s="4" t="inlineStr">
+      <c r="B161" s="5" t="inlineStr">
         <is>
           <t>isResolved</t>
         </is>
       </c>
-      <c r="C161" s="4" t="inlineStr">
+      <c r="C161" s="5" t="inlineStr">
         <is>
           <t>Boolean</t>
         </is>
       </c>
-      <c r="D161" s="4" t="inlineStr"/>
-      <c r="E161" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F161" s="4" t="inlineStr"/>
-      <c r="G161" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H161" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+      <c r="D161" s="5" t="inlineStr"/>
+      <c r="E161" s="5" t="inlineStr">
+        <is>
+          <t>Out of v1 scope</t>
+        </is>
+      </c>
+      <c r="F161" s="5" t="inlineStr"/>
+      <c r="G161" s="5" t="inlineStr"/>
+      <c r="H161" s="5" t="inlineStr">
+        <is>
+          <t>No corresponding purchase_orders field is marked needed for CoCre8 in the edited reference workbook.</t>
         </is>
       </c>
     </row>
     <row r="162">
-      <c r="A162" s="4" t="inlineStr">
+      <c r="A162" s="2" t="inlineStr">
         <is>
           <t>PurchaseOrders</t>
         </is>
       </c>
-      <c r="B162" s="4" t="inlineStr">
+      <c r="B162" s="2" t="inlineStr">
         <is>
           <t>partNumber</t>
         </is>
       </c>
-      <c r="C162" s="4" t="inlineStr">
+      <c r="C162" s="2" t="inlineStr">
         <is>
           <t>String</t>
         </is>
       </c>
-      <c r="D162" s="4" t="inlineStr"/>
-      <c r="E162" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F162" s="4" t="inlineStr"/>
-      <c r="G162" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H162" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+      <c r="D162" s="2" t="inlineStr"/>
+      <c r="E162" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="F162" s="2" t="inlineStr">
+        <is>
+          <t>SAP Service Layer SQLQueries:POR1.ItemCode</t>
+        </is>
+      </c>
+      <c r="G162" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H162" s="2" t="inlineStr">
+        <is>
+          <t>Populated in template CSV from confirmed live SAP Service Layer or allowed SPI source.</t>
         </is>
       </c>
     </row>
     <row r="163">
-      <c r="A163" s="4" t="inlineStr">
+      <c r="A163" s="2" t="inlineStr">
         <is>
           <t>PurchaseOrders</t>
         </is>
       </c>
-      <c r="B163" s="4" t="inlineStr">
+      <c r="B163" s="2" t="inlineStr">
         <is>
           <t>quantity</t>
         </is>
       </c>
-      <c r="C163" s="4" t="inlineStr">
+      <c r="C163" s="2" t="inlineStr">
         <is>
           <t>Double</t>
         </is>
       </c>
-      <c r="D163" s="4" t="inlineStr"/>
-      <c r="E163" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F163" s="4" t="inlineStr"/>
-      <c r="G163" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H163" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+      <c r="D163" s="2" t="inlineStr"/>
+      <c r="E163" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="F163" s="2" t="inlineStr">
+        <is>
+          <t>SAP Service Layer SQLQueries:POR1.Quantity</t>
+        </is>
+      </c>
+      <c r="G163" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H163" s="2" t="inlineStr">
+        <is>
+          <t>Populated in template CSV from confirmed live SAP Service Layer or allowed SPI source.</t>
         </is>
       </c>
     </row>
     <row r="164">
-      <c r="A164" s="4" t="inlineStr">
+      <c r="A164" s="2" t="inlineStr">
         <is>
           <t>PurchaseOrders</t>
         </is>
       </c>
-      <c r="B164" s="4" t="inlineStr">
+      <c r="B164" s="2" t="inlineStr">
         <is>
           <t>lineCost</t>
         </is>
       </c>
-      <c r="C164" s="4" t="inlineStr">
+      <c r="C164" s="2" t="inlineStr">
         <is>
           <t>Double</t>
         </is>
       </c>
-      <c r="D164" s="4" t="inlineStr"/>
-      <c r="E164" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F164" s="4" t="inlineStr"/>
-      <c r="G164" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H164" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+      <c r="D164" s="2" t="inlineStr"/>
+      <c r="E164" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="F164" s="2" t="inlineStr">
+        <is>
+          <t>SAP Service Layer SQLQueries:POR1.LineTotal</t>
+        </is>
+      </c>
+      <c r="G164" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H164" s="2" t="inlineStr">
+        <is>
+          <t>Populated in template CSV from confirmed live SAP Service Layer or allowed SPI source.</t>
         </is>
       </c>
     </row>
     <row r="165">
-      <c r="A165" s="4" t="inlineStr">
+      <c r="A165" s="2" t="inlineStr">
         <is>
           <t>PurchaseOrders</t>
         </is>
       </c>
-      <c r="B165" s="4" t="inlineStr">
+      <c r="B165" s="2" t="inlineStr">
         <is>
           <t>quantityReceived</t>
         </is>
       </c>
-      <c r="C165" s="4" t="inlineStr">
+      <c r="C165" s="2" t="inlineStr">
         <is>
           <t>Double</t>
         </is>
       </c>
-      <c r="D165" s="4" t="inlineStr"/>
-      <c r="E165" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F165" s="4" t="inlineStr"/>
-      <c r="G165" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H165" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+      <c r="D165" s="2" t="inlineStr"/>
+      <c r="E165" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="F165" s="2" t="inlineStr">
+        <is>
+          <t>SAP Service Layer SQLQueries:PDN1.Quantity summed by PO line</t>
+        </is>
+      </c>
+      <c r="G165" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H165" s="2" t="inlineStr">
+        <is>
+          <t>Populated in template CSV from confirmed live SAP Service Layer or allowed SPI source.</t>
         </is>
       </c>
     </row>
     <row r="166">
-      <c r="A166" s="4" t="inlineStr">
+      <c r="A166" s="2" t="inlineStr">
         <is>
           <t>PurchaseOrders</t>
         </is>
       </c>
-      <c r="B166" s="4" t="inlineStr">
+      <c r="B166" s="2" t="inlineStr">
         <is>
           <t>receivedDateTime</t>
         </is>
       </c>
-      <c r="C166" s="4" t="inlineStr">
+      <c r="C166" s="2" t="inlineStr">
         <is>
           <t>Datetime</t>
         </is>
       </c>
-      <c r="D166" s="4" t="inlineStr"/>
-      <c r="E166" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="F166" s="4" t="inlineStr"/>
-      <c r="G166" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H166" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
+      <c r="D166" s="2" t="inlineStr"/>
+      <c r="E166" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="F166" s="2" t="inlineStr">
+        <is>
+          <t>SAP Service Layer SQLQueries:OPDN.DocDate max by PO line</t>
+        </is>
+      </c>
+      <c r="G166" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H166" s="2" t="inlineStr">
+        <is>
+          <t>Populated in template CSV from confirmed live SAP Service Layer or allowed SPI source.</t>
         </is>
       </c>
     </row>
@@ -19185,7 +19217,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G249"/>
+  <dimension ref="A1:G235"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -27562,7 +27594,7 @@
     <row r="227">
       <c r="A227" s="4" t="inlineStr">
         <is>
-          <t>purchaseOrderNumber</t>
+          <t>demandStatus</t>
         </is>
       </c>
       <c r="B227" s="4" t="inlineStr">
@@ -27582,7 +27614,7 @@
       </c>
       <c r="E227" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PurchaseOrders.purchaseOrderNumber?</t>
+          <t>What confirmed CoCre8/SAP source should populate PurchaseOrders.demandStatus?</t>
         </is>
       </c>
       <c r="F227" s="4" t="inlineStr">
@@ -27599,12 +27631,12 @@
     <row r="228">
       <c r="A228" s="4" t="inlineStr">
         <is>
-          <t>purchaseOrderStatus</t>
+          <t>partTypeCode</t>
         </is>
       </c>
       <c r="B228" s="4" t="inlineStr">
         <is>
-          <t>PurchaseOrders</t>
+          <t>PartTypes</t>
         </is>
       </c>
       <c r="C228" s="4" t="inlineStr">
@@ -27619,7 +27651,7 @@
       </c>
       <c r="E228" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PurchaseOrders.purchaseOrderStatus?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartTypes.partTypeCode?</t>
         </is>
       </c>
       <c r="F228" s="4" t="inlineStr">
@@ -27636,12 +27668,12 @@
     <row r="229">
       <c r="A229" s="4" t="inlineStr">
         <is>
-          <t>creationDateTime</t>
+          <t>description</t>
         </is>
       </c>
       <c r="B229" s="4" t="inlineStr">
         <is>
-          <t>PurchaseOrders</t>
+          <t>PartTypes</t>
         </is>
       </c>
       <c r="C229" s="4" t="inlineStr">
@@ -27656,7 +27688,7 @@
       </c>
       <c r="E229" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PurchaseOrders.creationDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate PartTypes.description?</t>
         </is>
       </c>
       <c r="F229" s="4" t="inlineStr">
@@ -27673,12 +27705,12 @@
     <row r="230">
       <c r="A230" s="4" t="inlineStr">
         <is>
-          <t>approvalDateTime</t>
+          <t>partNumber</t>
         </is>
       </c>
       <c r="B230" s="4" t="inlineStr">
         <is>
-          <t>PurchaseOrders</t>
+          <t>Yields</t>
         </is>
       </c>
       <c r="C230" s="4" t="inlineStr">
@@ -27693,7 +27725,7 @@
       </c>
       <c r="E230" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PurchaseOrders.approvalDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate Yields.partNumber?</t>
         </is>
       </c>
       <c r="F230" s="4" t="inlineStr">
@@ -27710,12 +27742,12 @@
     <row r="231">
       <c r="A231" s="4" t="inlineStr">
         <is>
-          <t>toWarehouseId</t>
+          <t>unitOfMeasure</t>
         </is>
       </c>
       <c r="B231" s="4" t="inlineStr">
         <is>
-          <t>PurchaseOrders</t>
+          <t>Yields</t>
         </is>
       </c>
       <c r="C231" s="4" t="inlineStr">
@@ -27730,7 +27762,7 @@
       </c>
       <c r="E231" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PurchaseOrders.toWarehouseId?</t>
+          <t>What confirmed CoCre8/SAP source should populate Yields.unitOfMeasure?</t>
         </is>
       </c>
       <c r="F231" s="4" t="inlineStr">
@@ -27747,12 +27779,12 @@
     <row r="232">
       <c r="A232" s="4" t="inlineStr">
         <is>
-          <t>vendorId</t>
+          <t>yield</t>
         </is>
       </c>
       <c r="B232" s="4" t="inlineStr">
         <is>
-          <t>PurchaseOrders</t>
+          <t>Yields</t>
         </is>
       </c>
       <c r="C232" s="4" t="inlineStr">
@@ -27767,7 +27799,7 @@
       </c>
       <c r="E232" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PurchaseOrders.vendorId?</t>
+          <t>What confirmed CoCre8/SAP source should populate Yields.yield?</t>
         </is>
       </c>
       <c r="F232" s="4" t="inlineStr">
@@ -27784,12 +27816,12 @@
     <row r="233">
       <c r="A233" s="4" t="inlineStr">
         <is>
-          <t>demandStatus</t>
+          <t>warehouseId</t>
         </is>
       </c>
       <c r="B233" s="4" t="inlineStr">
         <is>
-          <t>PurchaseOrders</t>
+          <t>WarehouseExclusions</t>
         </is>
       </c>
       <c r="C233" s="4" t="inlineStr">
@@ -27804,7 +27836,7 @@
       </c>
       <c r="E233" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PurchaseOrders.demandStatus?</t>
+          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.warehouseId?</t>
         </is>
       </c>
       <c r="F233" s="4" t="inlineStr">
@@ -27821,12 +27853,12 @@
     <row r="234">
       <c r="A234" s="4" t="inlineStr">
         <is>
-          <t>customerId</t>
+          <t>exclusionType</t>
         </is>
       </c>
       <c r="B234" s="4" t="inlineStr">
         <is>
-          <t>PurchaseOrders</t>
+          <t>WarehouseExclusions</t>
         </is>
       </c>
       <c r="C234" s="4" t="inlineStr">
@@ -27841,7 +27873,7 @@
       </c>
       <c r="E234" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PurchaseOrders.customerId?</t>
+          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.exclusionType?</t>
         </is>
       </c>
       <c r="F234" s="4" t="inlineStr">
@@ -27858,12 +27890,12 @@
     <row r="235">
       <c r="A235" s="4" t="inlineStr">
         <is>
-          <t>requestTicketDateTime</t>
+          <t>exclusion</t>
         </is>
       </c>
       <c r="B235" s="4" t="inlineStr">
         <is>
-          <t>PurchaseOrders</t>
+          <t>WarehouseExclusions</t>
         </is>
       </c>
       <c r="C235" s="4" t="inlineStr">
@@ -27878,7 +27910,7 @@
       </c>
       <c r="E235" s="4" t="inlineStr">
         <is>
-          <t>What confirmed CoCre8/SAP source should populate PurchaseOrders.requestTicketDateTime?</t>
+          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.exclusion?</t>
         </is>
       </c>
       <c r="F235" s="4" t="inlineStr">
@@ -27892,526 +27924,8 @@
         </is>
       </c>
     </row>
-    <row r="236">
-      <c r="A236" s="4" t="inlineStr">
-        <is>
-          <t>isResolved</t>
-        </is>
-      </c>
-      <c r="B236" s="4" t="inlineStr">
-        <is>
-          <t>PurchaseOrders</t>
-        </is>
-      </c>
-      <c r="C236" s="4" t="inlineStr">
-        <is>
-          <t>Planning V2 template</t>
-        </is>
-      </c>
-      <c r="D236" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="E236" s="4" t="inlineStr">
-        <is>
-          <t>What confirmed CoCre8/SAP source should populate PurchaseOrders.isResolved?</t>
-        </is>
-      </c>
-      <c r="F236" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP Service Layer first; only use external/manual source if SAP cannot supply it.</t>
-        </is>
-      </c>
-      <c r="G236" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="237">
-      <c r="A237" s="4" t="inlineStr">
-        <is>
-          <t>partNumber</t>
-        </is>
-      </c>
-      <c r="B237" s="4" t="inlineStr">
-        <is>
-          <t>PurchaseOrders</t>
-        </is>
-      </c>
-      <c r="C237" s="4" t="inlineStr">
-        <is>
-          <t>Planning V2 template</t>
-        </is>
-      </c>
-      <c r="D237" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="E237" s="4" t="inlineStr">
-        <is>
-          <t>What confirmed CoCre8/SAP source should populate PurchaseOrders.partNumber?</t>
-        </is>
-      </c>
-      <c r="F237" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP Service Layer first; only use external/manual source if SAP cannot supply it.</t>
-        </is>
-      </c>
-      <c r="G237" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="238">
-      <c r="A238" s="4" t="inlineStr">
-        <is>
-          <t>quantity</t>
-        </is>
-      </c>
-      <c r="B238" s="4" t="inlineStr">
-        <is>
-          <t>PurchaseOrders</t>
-        </is>
-      </c>
-      <c r="C238" s="4" t="inlineStr">
-        <is>
-          <t>Planning V2 template</t>
-        </is>
-      </c>
-      <c r="D238" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="E238" s="4" t="inlineStr">
-        <is>
-          <t>What confirmed CoCre8/SAP source should populate PurchaseOrders.quantity?</t>
-        </is>
-      </c>
-      <c r="F238" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP Service Layer first; only use external/manual source if SAP cannot supply it.</t>
-        </is>
-      </c>
-      <c r="G238" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="239">
-      <c r="A239" s="4" t="inlineStr">
-        <is>
-          <t>lineCost</t>
-        </is>
-      </c>
-      <c r="B239" s="4" t="inlineStr">
-        <is>
-          <t>PurchaseOrders</t>
-        </is>
-      </c>
-      <c r="C239" s="4" t="inlineStr">
-        <is>
-          <t>Planning V2 template</t>
-        </is>
-      </c>
-      <c r="D239" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="E239" s="4" t="inlineStr">
-        <is>
-          <t>What confirmed CoCre8/SAP source should populate PurchaseOrders.lineCost?</t>
-        </is>
-      </c>
-      <c r="F239" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP Service Layer first; only use external/manual source if SAP cannot supply it.</t>
-        </is>
-      </c>
-      <c r="G239" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="240">
-      <c r="A240" s="4" t="inlineStr">
-        <is>
-          <t>quantityReceived</t>
-        </is>
-      </c>
-      <c r="B240" s="4" t="inlineStr">
-        <is>
-          <t>PurchaseOrders</t>
-        </is>
-      </c>
-      <c r="C240" s="4" t="inlineStr">
-        <is>
-          <t>Planning V2 template</t>
-        </is>
-      </c>
-      <c r="D240" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="E240" s="4" t="inlineStr">
-        <is>
-          <t>What confirmed CoCre8/SAP source should populate PurchaseOrders.quantityReceived?</t>
-        </is>
-      </c>
-      <c r="F240" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP Service Layer first; only use external/manual source if SAP cannot supply it.</t>
-        </is>
-      </c>
-      <c r="G240" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="241">
-      <c r="A241" s="4" t="inlineStr">
-        <is>
-          <t>receivedDateTime</t>
-        </is>
-      </c>
-      <c r="B241" s="4" t="inlineStr">
-        <is>
-          <t>PurchaseOrders</t>
-        </is>
-      </c>
-      <c r="C241" s="4" t="inlineStr">
-        <is>
-          <t>Planning V2 template</t>
-        </is>
-      </c>
-      <c r="D241" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="E241" s="4" t="inlineStr">
-        <is>
-          <t>What confirmed CoCre8/SAP source should populate PurchaseOrders.receivedDateTime?</t>
-        </is>
-      </c>
-      <c r="F241" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP Service Layer first; only use external/manual source if SAP cannot supply it.</t>
-        </is>
-      </c>
-      <c r="G241" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="242">
-      <c r="A242" s="4" t="inlineStr">
-        <is>
-          <t>partTypeCode</t>
-        </is>
-      </c>
-      <c r="B242" s="4" t="inlineStr">
-        <is>
-          <t>PartTypes</t>
-        </is>
-      </c>
-      <c r="C242" s="4" t="inlineStr">
-        <is>
-          <t>Planning V2 template</t>
-        </is>
-      </c>
-      <c r="D242" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="E242" s="4" t="inlineStr">
-        <is>
-          <t>What confirmed CoCre8/SAP source should populate PartTypes.partTypeCode?</t>
-        </is>
-      </c>
-      <c r="F242" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP Service Layer first; only use external/manual source if SAP cannot supply it.</t>
-        </is>
-      </c>
-      <c r="G242" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="243">
-      <c r="A243" s="4" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="B243" s="4" t="inlineStr">
-        <is>
-          <t>PartTypes</t>
-        </is>
-      </c>
-      <c r="C243" s="4" t="inlineStr">
-        <is>
-          <t>Planning V2 template</t>
-        </is>
-      </c>
-      <c r="D243" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="E243" s="4" t="inlineStr">
-        <is>
-          <t>What confirmed CoCre8/SAP source should populate PartTypes.description?</t>
-        </is>
-      </c>
-      <c r="F243" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP Service Layer first; only use external/manual source if SAP cannot supply it.</t>
-        </is>
-      </c>
-      <c r="G243" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="244">
-      <c r="A244" s="4" t="inlineStr">
-        <is>
-          <t>partNumber</t>
-        </is>
-      </c>
-      <c r="B244" s="4" t="inlineStr">
-        <is>
-          <t>Yields</t>
-        </is>
-      </c>
-      <c r="C244" s="4" t="inlineStr">
-        <is>
-          <t>Planning V2 template</t>
-        </is>
-      </c>
-      <c r="D244" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="E244" s="4" t="inlineStr">
-        <is>
-          <t>What confirmed CoCre8/SAP source should populate Yields.partNumber?</t>
-        </is>
-      </c>
-      <c r="F244" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP Service Layer first; only use external/manual source if SAP cannot supply it.</t>
-        </is>
-      </c>
-      <c r="G244" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="245">
-      <c r="A245" s="4" t="inlineStr">
-        <is>
-          <t>unitOfMeasure</t>
-        </is>
-      </c>
-      <c r="B245" s="4" t="inlineStr">
-        <is>
-          <t>Yields</t>
-        </is>
-      </c>
-      <c r="C245" s="4" t="inlineStr">
-        <is>
-          <t>Planning V2 template</t>
-        </is>
-      </c>
-      <c r="D245" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="E245" s="4" t="inlineStr">
-        <is>
-          <t>What confirmed CoCre8/SAP source should populate Yields.unitOfMeasure?</t>
-        </is>
-      </c>
-      <c r="F245" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP Service Layer first; only use external/manual source if SAP cannot supply it.</t>
-        </is>
-      </c>
-      <c r="G245" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="246">
-      <c r="A246" s="4" t="inlineStr">
-        <is>
-          <t>yield</t>
-        </is>
-      </c>
-      <c r="B246" s="4" t="inlineStr">
-        <is>
-          <t>Yields</t>
-        </is>
-      </c>
-      <c r="C246" s="4" t="inlineStr">
-        <is>
-          <t>Planning V2 template</t>
-        </is>
-      </c>
-      <c r="D246" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="E246" s="4" t="inlineStr">
-        <is>
-          <t>What confirmed CoCre8/SAP source should populate Yields.yield?</t>
-        </is>
-      </c>
-      <c r="F246" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP Service Layer first; only use external/manual source if SAP cannot supply it.</t>
-        </is>
-      </c>
-      <c r="G246" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="247">
-      <c r="A247" s="4" t="inlineStr">
-        <is>
-          <t>warehouseId</t>
-        </is>
-      </c>
-      <c r="B247" s="4" t="inlineStr">
-        <is>
-          <t>WarehouseExclusions</t>
-        </is>
-      </c>
-      <c r="C247" s="4" t="inlineStr">
-        <is>
-          <t>Planning V2 template</t>
-        </is>
-      </c>
-      <c r="D247" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="E247" s="4" t="inlineStr">
-        <is>
-          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.warehouseId?</t>
-        </is>
-      </c>
-      <c r="F247" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP Service Layer first; only use external/manual source if SAP cannot supply it.</t>
-        </is>
-      </c>
-      <c r="G247" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="248">
-      <c r="A248" s="4" t="inlineStr">
-        <is>
-          <t>exclusionType</t>
-        </is>
-      </c>
-      <c r="B248" s="4" t="inlineStr">
-        <is>
-          <t>WarehouseExclusions</t>
-        </is>
-      </c>
-      <c r="C248" s="4" t="inlineStr">
-        <is>
-          <t>Planning V2 template</t>
-        </is>
-      </c>
-      <c r="D248" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="E248" s="4" t="inlineStr">
-        <is>
-          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.exclusionType?</t>
-        </is>
-      </c>
-      <c r="F248" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP Service Layer first; only use external/manual source if SAP cannot supply it.</t>
-        </is>
-      </c>
-      <c r="G248" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="249">
-      <c r="A249" s="4" t="inlineStr">
-        <is>
-          <t>exclusion</t>
-        </is>
-      </c>
-      <c r="B249" s="4" t="inlineStr">
-        <is>
-          <t>WarehouseExclusions</t>
-        </is>
-      </c>
-      <c r="C249" s="4" t="inlineStr">
-        <is>
-          <t>Planning V2 template</t>
-        </is>
-      </c>
-      <c r="D249" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP first</t>
-        </is>
-      </c>
-      <c r="E249" s="4" t="inlineStr">
-        <is>
-          <t>What confirmed CoCre8/SAP source should populate WarehouseExclusions.exclusion?</t>
-        </is>
-      </c>
-      <c r="F249" s="4" t="inlineStr">
-        <is>
-          <t>Investigate SAP Service Layer first; only use external/manual source if SAP cannot supply it.</t>
-        </is>
-      </c>
-      <c r="G249" s="4" t="inlineStr">
-        <is>
-          <t>Left blank in generated template CSV until source and semantics are confirmed.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:G249"/>
+  <autoFilter ref="A1:G235"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -29187,29 +28701,29 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="4" t="inlineStr">
+      <c r="A30" s="3" t="inlineStr">
         <is>
           <t>PurchaseOrders</t>
         </is>
       </c>
-      <c r="B30" s="4" t="inlineStr">
+      <c r="B30" s="3" t="inlineStr">
         <is>
           <t>PurchaseOrders.csv</t>
         </is>
       </c>
-      <c r="C30" s="4" t="inlineStr">
-        <is>
-          <t>Pending/header only</t>
-        </is>
-      </c>
-      <c r="D30" s="4" t="inlineStr">
-        <is>
-          <t>purchaseOrderNumber, purchaseOrderStatus, creationDateTime, approvalDateTime, toWarehouseId, vendorId, demandStatus, customerId, requestTicketDateTime, isResolved, partNumber, quantity, lineCost, quantityReceived, receivedDateTime</t>
-        </is>
-      </c>
-      <c r="E30" s="4" t="inlineStr">
-        <is>
-          <t>purchaseOrderNumber; purchaseOrderStatus; creationDateTime; approvalDateTime; toWarehouseId; vendorId; demandStatus; customerId; requestTicketDateTime; isResolved; partNumber; quantity; lineCost; quantityReceived; receivedDateTime</t>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>purchaseOrderNumber, purchaseOrderStatus, creationDateTime, approvalDateTime, toWarehouseId, vendorId, demandStatus, partNumber, quantity, lineCost, quantityReceived, receivedDateTime</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>demandStatus</t>
         </is>
       </c>
     </row>

</xml_diff>